<commit_message>
Clarify company review dates, evidence scope and Excel sources
</commit_message>
<xml_diff>
--- a/samples/lly_liquidity.xlsx
+++ b/samples/lly_liquidity.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding conclusion" sheetId="1" r:id="Rf70c54d8804b432d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt and liquidity" sheetId="2" r:id="R39aa0010726840c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repayment review" sheetId="3" r:id="R9b0003417e5c473f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="4" r:id="R34b2559cf224497e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="5" r:id="Ra50cf1abecf44321"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding conclusion" sheetId="1" r:id="Rc1d020c4a509471e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt and liquidity" sheetId="2" r:id="R8a17fbeb69d54df2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repayment review" sheetId="3" r:id="R54d37a84a18f420a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="4" r:id="Rb86a2bfa21ba4fb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="5" r:id="Rf6d05661dade4526"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1038,7 +1038,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R25e97008a7a949ab"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8704586239434e68"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2863,13 +2863,13 @@
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B50" s="140" t="str">
-        <x:v>Saved filings only</x:v>
+        <x:v>Financing index through Oct 15, 2026</x:v>
       </x:c>
       <x:c r="C50" s="118" t="str">
-        <x:v>10-K; 10-Q; Aug 5 Ex. 99.1</x:v>
+        <x:v>10-K; 10-Q; earnings and financing documents</x:v>
       </x:c>
       <x:c r="D50" s="18" t="str">
-        <x:v>Not a complete SEC filing inventory. No combined total of commitments, milestones, capex plans or debt.</x:v>
+        <x:v>SEC financing candidates screened through October 15. Not a complete review of all liability notes. No combined obligations total.</x:v>
       </x:c>
       <x:c r="E50" s="4"/>
       <x:c r="F50" s="4"/>
@@ -3613,7 +3613,7 @@
     <x:mergeCell ref="A96:D96"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R648b8cfda5fc4258"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf433d9363a34e67"/>
 </x:worksheet>
 </file>
 
@@ -9141,7 +9141,7 @@
         <x:v>0000059478-26-000081</x:v>
       </x:c>
       <x:c r="D115" s="16" t="str">
-        <x:v>pp. 7–8, 12–14, 17, 23, 31</x:v>
+        <x:v>Operations p. 5; segment Note 11 p. 23</x:v>
       </x:c>
       <x:c r="L115" s="173" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/59478/000005947826000081/lly-20260630.htm</x:v>
@@ -9158,7 +9158,7 @@
         <x:v>0000059478-26-000013</x:v>
       </x:c>
       <x:c r="D116" s="18" t="str">
-        <x:v>pp. 51, 57, 76–77</x:v>
+        <x:v>Operations p. 57; Borrowings Note 11 p. 77</x:v>
       </x:c>
       <x:c r="L116" s="174" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/59478/000005947826000013/lly-20251231.htm</x:v>
@@ -9189,12 +9189,12 @@
         <x:v>Source</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="70" customHeight="1">
+    <x:row r="2" ht="100" customHeight="1">
       <x:c r="A2" s="25" t="str">
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B2" s="116" t="str">
-        <x:v>Lilly only. Checked snapshot October 14, 2026. Financial statements dated June 30, 2026. Not investment advice.</x:v>
+        <x:v>Lilly only. Balance-sheet facts checked October 14, 2026; financing and interest reviewed October 15; funding interpretation checked October 16. Financial statements dated June 30. Not investment advice.</x:v>
       </x:c>
       <x:c r="C2" s="16" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/59478/000005947826000081/lly-20260630.htm</x:v>
@@ -9217,7 +9217,7 @@
         <x:v>Fiscal year + current YTD − prior YTD. Capital spending uses Lilly’s checked other-PP&amp;E tag. FCF excludes acquisitions, dividends and other cash uses.</x:v>
       </x:c>
       <x:c r="C4" s="16" t="str">
-        <x:v>docs/pilot_cashflow_reconciliation.md</x:v>
+        <x:v>https://github.com/jackconnolly1000-ux/sec-filing-research-terminal/blob/main/docs/pilot_cashflow_reconciliation.md</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="70" customHeight="1">
@@ -9228,7 +9228,7 @@
         <x:v>Balance-sheet current and noncurrent borrowing are added once. Fair-value table carrying amounts are not added again.</x:v>
       </x:c>
       <x:c r="C5" s="16" t="str">
-        <x:v>docs/pilot_evidence_lly.md</x:v>
+        <x:v>https://github.com/jackconnolly1000-ux/sec-filing-research-terminal/blob/main/docs/pilot_evidence_lly.md</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="70" customHeight="1">
@@ -9250,7 +9250,7 @@
         <x:v>Repayment review uses exact H1 cash flows and historical annual carrying-debt buckets. Future coverage remains Unavailable. Text disclosures are identified separately; source hashes and dimensions are in Data.</x:v>
       </x:c>
       <x:c r="C7" s="16" t="str">
-        <x:v>docs/lly_liquidity_review.md</x:v>
+        <x:v>https://github.com/jackconnolly1000-ux/sec-filing-research-terminal/blob/main/docs/lly_liquidity_review.md</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="95" customHeight="1">
@@ -9283,7 +9283,7 @@
         <x:v>Series rates and maturities come from the final prospectus and certificates, corroborated by the completed offering. An 8-K coupon conflict is flagged; the corroborated 2029 fixed rate is 4.150%.</x:v>
       </x:c>
       <x:c r="C10" s="18" t="str">
-        <x:v>docs/lly_financing_audit.md</x:v>
+        <x:v>https://github.com/jackconnolly1000-ux/sec-filing-research-terminal/blob/main/docs/lly_financing_audit.md</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="100" customHeight="1">
@@ -9294,7 +9294,7 @@
         <x:v>Derived TTM operating income / reported interest expense. FY + current H1 − prior H1; each operating-income period reconciles to pretax less tagged nonoperating income (expense).</x:v>
       </x:c>
       <x:c r="C11" s="16" t="str">
-        <x:v>docs/lly_interest_coverage.md</x:v>
+        <x:v>https://github.com/jackconnolly1000-ux/sec-filing-research-terminal/blob/main/docs/lly_interest_coverage.md</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="100" customHeight="1">

</xml_diff>

<commit_message>
Separate borrowing and dated lease balances
</commit_message>
<xml_diff>
--- a/samples/lly_liquidity.xlsx
+++ b/samples/lly_liquidity.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding conclusion" sheetId="1" r:id="Rc1d020c4a509471e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt and liquidity" sheetId="2" r:id="R8a17fbeb69d54df2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repayment review" sheetId="3" r:id="R54d37a84a18f420a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="4" r:id="Rb86a2bfa21ba4fb8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="5" r:id="Rf6d05661dade4526"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding conclusion" sheetId="1" r:id="R0690a579cb1f471b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Borrowing and leases" sheetId="2" r:id="R68a141c45d2142da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt and liquidity" sheetId="3" r:id="Re57f25ff60eb4c9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repayment review" sheetId="4" r:id="R53f5ac129a90469f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="5" r:id="R776c91b13bb947d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="6" r:id="R6f66b36fb08f4c06"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -371,7 +372,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="179">
+  <x:cellXfs count="196">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -840,6 +841,57 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="13" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="17" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1038,7 +1090,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8704586239434e68"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R44aeeb1f676e41f0"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1381,6 +1433,286 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="42" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="21" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="38" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="72" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="12" customHeight="1">
+      <x:c r="A1" s="4"/>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+    </x:row>
+    <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" s="7" t="str">
+        <x:v>Eli Lilly and Company borrowing and leases</x:v>
+      </x:c>
+      <x:c r="B2" s="4"/>
+      <x:c r="C2" s="4"/>
+      <x:c r="D2" s="4"/>
+      <x:c r="E2" s="4"/>
+    </x:row>
+    <x:row r="3" ht="25" customHeight="1">
+      <x:c r="A3" s="8" t="str">
+        <x:v>Amounts in USD millions. Each balance retains its own date. Baseline borrowing excludes leases.</x:v>
+      </x:c>
+      <x:c r="B3" s="4"/>
+      <x:c r="C3" s="4"/>
+      <x:c r="D3" s="4"/>
+      <x:c r="E3" s="4"/>
+    </x:row>
+    <x:row r="4" ht="12" customHeight="1">
+      <x:c r="A4" s="4"/>
+      <x:c r="B4" s="4"/>
+      <x:c r="C4" s="4"/>
+      <x:c r="D4" s="4"/>
+      <x:c r="E4" s="4"/>
+    </x:row>
+    <x:row r="5" ht="28" customHeight="1">
+      <x:c r="A5" s="13" t="str">
+        <x:v>Borrowing component</x:v>
+      </x:c>
+      <x:c r="B5" s="103" t="str">
+        <x:v>USD millions</x:v>
+      </x:c>
+      <x:c r="C5" s="103" t="str">
+        <x:v>As of</x:v>
+      </x:c>
+      <x:c r="D5" s="103" t="str">
+        <x:v>Source / filing</x:v>
+      </x:c>
+      <x:c r="E5" s="14" t="str">
+        <x:v>Basis</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="25" t="str">
+        <x:v>Current borrowing</x:v>
+      </x:c>
+      <x:c r="B6" s="81" t="n">
+        <x:f>IF(ISNUMBER('Data'!B120),'Data'!B120,NA())</x:f>
+        <x:v>7050000000</x:v>
+      </x:c>
+      <x:c r="C6" s="82" t="d">
+        <x:v>2026-06-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D6" s="116" t="str">
+        <x:v>10-Q balance sheet, p. 7; filed 2026-08-05</x:v>
+      </x:c>
+      <x:c r="E6" s="16" t="str">
+        <x:v>Short-term borrowings and current maturities of long-term debt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="25" t="str">
+        <x:v>Noncurrent borrowing</x:v>
+      </x:c>
+      <x:c r="B7" s="81" t="n">
+        <x:f>IF(ISNUMBER('Data'!B121),'Data'!B121,NA())</x:f>
+        <x:v>47858000000</x:v>
+      </x:c>
+      <x:c r="C7" s="82" t="d">
+        <x:v>2026-06-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D7" s="116" t="str">
+        <x:v>10-Q balance sheet, p. 7; filed 2026-08-05</x:v>
+      </x:c>
+      <x:c r="E7" s="16" t="str">
+        <x:v>Long-term debt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="130" t="str">
+        <x:v>Baseline gross debt</x:v>
+      </x:c>
+      <x:c r="B8" s="134" t="n">
+        <x:f>SUM(B6:B7)</x:f>
+        <x:v>54908000000</x:v>
+      </x:c>
+      <x:c r="C8" s="195" t="d">
+        <x:v>2026-06-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D8" s="132" t="str">
+        <x:v>Derived from the components above</x:v>
+      </x:c>
+      <x:c r="E8" s="133" t="str">
+        <x:v>Carrying amount; excludes leases.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="12" customHeight="1">
+      <x:c r="A9" s="4"/>
+      <x:c r="B9" s="135"/>
+      <x:c r="C9" s="60"/>
+      <x:c r="D9" s="4"/>
+      <x:c r="E9" s="4"/>
+    </x:row>
+    <x:row r="10" ht="58" customHeight="1">
+      <x:c r="A10" s="4" t="str">
+        <x:v>Borrowing scope</x:v>
+      </x:c>
+      <x:c r="B10" s="135"/>
+      <x:c r="C10" s="60"/>
+      <x:c r="D10" s="4"/>
+      <x:c r="E10" s="4" t="str">
+        <x:v>Current borrowing includes short-term borrowings and current maturities. The Note 8 fair-value carrying amounts describe the same debt and are not added.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="12" customHeight="1">
+      <x:c r="A11" s="4"/>
+      <x:c r="B11" s="135"/>
+      <x:c r="C11" s="60"/>
+      <x:c r="D11" s="4"/>
+      <x:c r="E11" s="4"/>
+    </x:row>
+    <x:row r="12" ht="12" customHeight="1">
+      <x:c r="A12" s="4"/>
+      <x:c r="B12" s="135"/>
+      <x:c r="C12" s="60"/>
+      <x:c r="D12" s="4"/>
+      <x:c r="E12" s="4"/>
+    </x:row>
+    <x:row r="13" ht="28" customHeight="1">
+      <x:c r="A13" s="13" t="str">
+        <x:v>Lease liability / commitment</x:v>
+      </x:c>
+      <x:c r="B13" s="136" t="str">
+        <x:v>USD millions</x:v>
+      </x:c>
+      <x:c r="C13" s="188" t="str">
+        <x:v>As of</x:v>
+      </x:c>
+      <x:c r="D13" s="103" t="str">
+        <x:v>Source / filing</x:v>
+      </x:c>
+      <x:c r="E13" s="14" t="str">
+        <x:v>Basis / Unavailable reason</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="42" customHeight="1">
+      <x:c r="A14" s="25" t="str">
+        <x:v>Lease liabilities at latest balance sheet</x:v>
+      </x:c>
+      <x:c r="B14" s="137" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="C14" s="82" t="d">
+        <x:v>2026-06-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D14" s="116" t="str">
+        <x:v>Checked 10-Q review</x:v>
+      </x:c>
+      <x:c r="E14" s="16" t="str">
+        <x:v>No lease liability amounts established in this 10-Q. Older amounts below are not substituted.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="42" customHeight="1">
+      <x:c r="A15" s="25" t="str">
+        <x:v>Operating lease liabilities — current</x:v>
+      </x:c>
+      <x:c r="B15" s="81" t="n">
+        <x:f>IF(ISNUMBER('Data'!B123),'Data'!B123,NA())</x:f>
+        <x:v>222000000</x:v>
+      </x:c>
+      <x:c r="C15" s="82" t="d">
+        <x:v>2025-12-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D15" s="116" t="str">
+        <x:v>10-K Note 10, p. 76; filed 2026-02-12</x:v>
+      </x:c>
+      <x:c r="E15" s="16" t="str">
+        <x:v>Recognized lease liability; excluded from baseline borrowing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="42" customHeight="1">
+      <x:c r="A16" s="25" t="str">
+        <x:v>Operating lease liabilities — noncurrent</x:v>
+      </x:c>
+      <x:c r="B16" s="81" t="n">
+        <x:f>IF(ISNUMBER('Data'!B124),'Data'!B124,NA())</x:f>
+        <x:v>1140000000</x:v>
+      </x:c>
+      <x:c r="C16" s="82" t="d">
+        <x:v>2025-12-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D16" s="116" t="str">
+        <x:v>10-K Note 10, p. 76; filed 2026-02-12</x:v>
+      </x:c>
+      <x:c r="E16" s="16" t="str">
+        <x:v>Recognized lease liability; excluded from baseline borrowing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="42" customHeight="1">
+      <x:c r="A17" s="107" t="str">
+        <x:v>Operating lease liabilities — total</x:v>
+      </x:c>
+      <x:c r="B17" s="112" t="n">
+        <x:f>B15+B16</x:f>
+        <x:v>1362000000</x:v>
+      </x:c>
+      <x:c r="C17" s="109" t="d">
+        <x:v>2025-12-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D17" s="126" t="str">
+        <x:v>10-K Note 10, p. 76</x:v>
+      </x:c>
+      <x:c r="E17" s="110" t="str">
+        <x:v>Derived current + noncurrent; no separately tagged total.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="42" customHeight="1">
+      <x:c r="A18" s="26" t="str">
+        <x:v>Finance lease liabilities</x:v>
+      </x:c>
+      <x:c r="B18" s="140" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="C18" s="87" t="d">
+        <x:v>2026-06-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D18" s="118" t="str">
+        <x:v>10-Q review; June amount not established</x:v>
+      </x:c>
+      <x:c r="E18" s="18" t="str">
+        <x:v>No checked June amount. The 10-K describes operating leases only; finance leases are not reported, which is not zero.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="12" customHeight="1">
+      <x:c r="A19" s="4"/>
+      <x:c r="B19" s="135"/>
+      <x:c r="C19" s="60"/>
+      <x:c r="D19" s="4"/>
+      <x:c r="E19" s="4"/>
+    </x:row>
+    <x:row r="20" ht="54" customHeight="1">
+      <x:c r="A20" s="157" t="str">
+        <x:v>Leases not yet commenced</x:v>
+      </x:c>
+      <x:c r="B20" s="189" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="C20" s="190" t="d">
+        <x:v>2026-06-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D20" s="191" t="str">
+        <x:v>Saved pilot evidence; 10-Q review</x:v>
+      </x:c>
+      <x:c r="E20" s="192" t="str">
+        <x:v>No checked amount for leases not yet commenced is established in the saved pilot evidence. Unavailable does not mean zero.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="42" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="29" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="73" hidden="0" customWidth="1"/>
@@ -2027,7 +2359,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -3613,11 +3945,11 @@
     <x:mergeCell ref="A96:D96"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf433d9363a34e67"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06119863eaed4991"/>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -9164,12 +9496,314 @@
         <x:v>https://www.sec.gov/Archives/edgar/data/59478/000005947826000013/lly-20251231.htm</x:v>
       </x:c>
     </x:row>
+    <x:row r="119" ht="78" customHeight="1">
+      <x:c r="A119" s="13" t="str">
+        <x:v>Input</x:v>
+      </x:c>
+      <x:c r="B119" s="103" t="str">
+        <x:v>USD millions</x:v>
+      </x:c>
+      <x:c r="C119" s="103" t="str">
+        <x:v>Period start</x:v>
+      </x:c>
+      <x:c r="D119" s="103" t="str">
+        <x:v>Period end</x:v>
+      </x:c>
+      <x:c r="E119" s="103" t="str">
+        <x:v>Form</x:v>
+      </x:c>
+      <x:c r="F119" s="103" t="str">
+        <x:v>Filed</x:v>
+      </x:c>
+      <x:c r="G119" s="103" t="str">
+        <x:v>Accession</x:v>
+      </x:c>
+      <x:c r="H119" s="103" t="str">
+        <x:v>Tag</x:v>
+      </x:c>
+      <x:c r="I119" s="103" t="str">
+        <x:v>Context</x:v>
+      </x:c>
+      <x:c r="J119" s="103" t="str">
+        <x:v>Scale</x:v>
+      </x:c>
+      <x:c r="K119" s="103" t="str">
+        <x:v>Decimals</x:v>
+      </x:c>
+      <x:c r="L119" s="103" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="M119" s="103" t="str">
+        <x:v>Filing location</x:v>
+      </x:c>
+      <x:c r="N119" s="103" t="str">
+        <x:v>Unavailable reason</x:v>
+      </x:c>
+      <x:c r="O119" s="14" t="str">
+        <x:v>Reviewed source SHA256</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="78" customHeight="1">
+      <x:c r="A120" s="25" t="str">
+        <x:v>Current borrowing</x:v>
+      </x:c>
+      <x:c r="B120" s="115" t="n">
+        <x:v>7050000000</x:v>
+      </x:c>
+      <x:c r="C120" s="116"/>
+      <x:c r="D120" s="82" t="d">
+        <x:v>2026-06-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E120" s="116" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F120" s="82" t="d">
+        <x:v>2026-08-05T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G120" s="116" t="str">
+        <x:v>0000059478-26-000081</x:v>
+      </x:c>
+      <x:c r="H120" s="116" t="str">
+        <x:v>us-gaap:DebtCurrent</x:v>
+      </x:c>
+      <x:c r="I120" s="116"/>
+      <x:c r="J120" s="116"/>
+      <x:c r="K120" s="116"/>
+      <x:c r="L120" s="116" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/59478/000005947826000081/lly-20260630.htm</x:v>
+      </x:c>
+      <x:c r="M120" s="116" t="str">
+        <x:v>10-Q balance sheet, p. 7</x:v>
+      </x:c>
+      <x:c r="N120" s="116" t="str"/>
+      <x:c r="O120" s="16" t="str"/>
+    </x:row>
+    <x:row r="121" ht="78" customHeight="1">
+      <x:c r="A121" s="25" t="str">
+        <x:v>Noncurrent borrowing</x:v>
+      </x:c>
+      <x:c r="B121" s="115" t="n">
+        <x:v>47858000000</x:v>
+      </x:c>
+      <x:c r="C121" s="116"/>
+      <x:c r="D121" s="82" t="d">
+        <x:v>2026-06-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E121" s="116" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F121" s="82" t="d">
+        <x:v>2026-08-05T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G121" s="116" t="str">
+        <x:v>0000059478-26-000081</x:v>
+      </x:c>
+      <x:c r="H121" s="116" t="str">
+        <x:v>us-gaap:LongTermDebtNoncurrent</x:v>
+      </x:c>
+      <x:c r="I121" s="116"/>
+      <x:c r="J121" s="116"/>
+      <x:c r="K121" s="116"/>
+      <x:c r="L121" s="116" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/59478/000005947826000081/lly-20260630.htm</x:v>
+      </x:c>
+      <x:c r="M121" s="116" t="str">
+        <x:v>10-Q balance sheet, p. 7</x:v>
+      </x:c>
+      <x:c r="N121" s="116" t="str"/>
+      <x:c r="O121" s="16" t="str"/>
+    </x:row>
+    <x:row r="122" ht="78" customHeight="1">
+      <x:c r="A122" s="25" t="str">
+        <x:v>Latest-date lease liabilities — Unavailable</x:v>
+      </x:c>
+      <x:c r="B122" s="115"/>
+      <x:c r="C122" s="116"/>
+      <x:c r="D122" s="82" t="d">
+        <x:v>2026-06-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E122" s="116" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F122" s="82" t="d">
+        <x:v>2026-08-05T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G122" s="116" t="str">
+        <x:v>0000059478-26-000081</x:v>
+      </x:c>
+      <x:c r="H122" s="116"/>
+      <x:c r="I122" s="116"/>
+      <x:c r="J122" s="116"/>
+      <x:c r="K122" s="116"/>
+      <x:c r="L122" s="116" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/59478/000005947826000081/lly-20260630.htm</x:v>
+      </x:c>
+      <x:c r="M122" s="116" t="str">
+        <x:v>10-Q balance sheet, p. 7</x:v>
+      </x:c>
+      <x:c r="N122" s="116" t="str">
+        <x:v>Latest-date lease liabilities Unavailable; no checked amount in the 10-Q.</x:v>
+      </x:c>
+      <x:c r="O122" s="16" t="str"/>
+    </x:row>
+    <x:row r="123" ht="78" customHeight="1">
+      <x:c r="A123" s="25" t="str">
+        <x:v>Operating lease liabilities — current</x:v>
+      </x:c>
+      <x:c r="B123" s="115" t="n">
+        <x:v>222000000</x:v>
+      </x:c>
+      <x:c r="C123" s="116"/>
+      <x:c r="D123" s="82" t="d">
+        <x:v>2025-12-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E123" s="116" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F123" s="82" t="d">
+        <x:v>2026-02-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G123" s="116" t="str">
+        <x:v>0000059478-26-000013</x:v>
+      </x:c>
+      <x:c r="H123" s="116" t="str">
+        <x:v>us-gaap:OperatingLeaseLiabilityCurrent</x:v>
+      </x:c>
+      <x:c r="I123" s="116" t="str">
+        <x:v>c-16</x:v>
+      </x:c>
+      <x:c r="J123" s="116" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K123" s="116" t="str">
+        <x:v>-6</x:v>
+      </x:c>
+      <x:c r="L123" s="116" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/59478/000005947826000013/lly-20251231.htm</x:v>
+      </x:c>
+      <x:c r="M123" s="116" t="str">
+        <x:v>10-K Note 10, p. 76</x:v>
+      </x:c>
+      <x:c r="N123" s="116" t="str"/>
+      <x:c r="O123" s="16" t="str">
+        <x:v>d45f8d1e0945df0b7b30254e96ff8c5dbd1df7d15b17c8ef7399c8e0206b7d7f</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="78" customHeight="1">
+      <x:c r="A124" s="25" t="str">
+        <x:v>Operating lease liabilities — noncurrent</x:v>
+      </x:c>
+      <x:c r="B124" s="115" t="n">
+        <x:v>1140000000</x:v>
+      </x:c>
+      <x:c r="C124" s="116"/>
+      <x:c r="D124" s="82" t="d">
+        <x:v>2025-12-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E124" s="116" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F124" s="82" t="d">
+        <x:v>2026-02-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G124" s="116" t="str">
+        <x:v>0000059478-26-000013</x:v>
+      </x:c>
+      <x:c r="H124" s="116" t="str">
+        <x:v>us-gaap:OperatingLeaseLiabilityNoncurrent</x:v>
+      </x:c>
+      <x:c r="I124" s="116" t="str">
+        <x:v>c-16</x:v>
+      </x:c>
+      <x:c r="J124" s="116" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K124" s="116" t="str">
+        <x:v>-6</x:v>
+      </x:c>
+      <x:c r="L124" s="116" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/59478/000005947826000013/lly-20251231.htm</x:v>
+      </x:c>
+      <x:c r="M124" s="116" t="str">
+        <x:v>10-K Note 10, p. 76</x:v>
+      </x:c>
+      <x:c r="N124" s="116" t="str"/>
+      <x:c r="O124" s="16" t="str">
+        <x:v>d45f8d1e0945df0b7b30254e96ff8c5dbd1df7d15b17c8ef7399c8e0206b7d7f</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="78" customHeight="1">
+      <x:c r="A125" s="25" t="str">
+        <x:v>Finance lease liabilities — requested date, Unavailable</x:v>
+      </x:c>
+      <x:c r="B125" s="115"/>
+      <x:c r="C125" s="116"/>
+      <x:c r="D125" s="82" t="d">
+        <x:v>2026-06-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E125" s="116" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F125" s="82" t="d">
+        <x:v>2026-08-05T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G125" s="116" t="str">
+        <x:v>0000059478-26-000081</x:v>
+      </x:c>
+      <x:c r="H125" s="116"/>
+      <x:c r="I125" s="116"/>
+      <x:c r="J125" s="116"/>
+      <x:c r="K125" s="116"/>
+      <x:c r="L125" s="116" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/59478/000005947826000081/lly-20260630.htm</x:v>
+      </x:c>
+      <x:c r="M125" s="116" t="str">
+        <x:v>10-Q review; June amount not established</x:v>
+      </x:c>
+      <x:c r="N125" s="116" t="str">
+        <x:v>No checked June amount. The 10-K describes operating leases only; finance leases are not reported, which is not zero.</x:v>
+      </x:c>
+      <x:c r="O125" s="16" t="str"/>
+    </x:row>
+    <x:row r="126" ht="78" customHeight="1">
+      <x:c r="A126" s="26" t="str">
+        <x:v>Leases not yet commenced — Unavailable</x:v>
+      </x:c>
+      <x:c r="B126" s="117"/>
+      <x:c r="C126" s="118"/>
+      <x:c r="D126" s="87" t="d">
+        <x:v>2026-06-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E126" s="118" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="F126" s="87" t="d">
+        <x:v>2026-08-05T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G126" s="118" t="str">
+        <x:v>0000059478-26-000081</x:v>
+      </x:c>
+      <x:c r="H126" s="118"/>
+      <x:c r="I126" s="118"/>
+      <x:c r="J126" s="118"/>
+      <x:c r="K126" s="118"/>
+      <x:c r="L126" s="118" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/59478/000005947826000081/lly-20260630.htm</x:v>
+      </x:c>
+      <x:c r="M126" s="118" t="str">
+        <x:v>Saved pilot evidence; 10-Q review</x:v>
+      </x:c>
+      <x:c r="N126" s="118" t="str">
+        <x:v>No checked amount for leases not yet commenced is established in the saved pilot evidence. Unavailable does not mean zero.</x:v>
+      </x:c>
+      <x:c r="O126" s="18" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -9308,6 +9942,17 @@
         <x:v>FY2025 10-K Note 11 p. 77; June 10-Q Note 11 p. 23</x:v>
       </x:c>
     </x:row>
+    <x:row r="13" ht="78" customHeight="1">
+      <x:c r="A13" s="157" t="str">
+        <x:v>Borrowing and leases</x:v>
+      </x:c>
+      <x:c r="B13" s="191" t="str">
+        <x:v>The Borrowing and leases sheet reconciles baseline borrowing and shows lease balances on their own dates. Unavailable means the amount was not established in the checked evidence. Leases never enter baseline debt or its ratios.</x:v>
+      </x:c>
+      <x:c r="C13" s="192" t="str">
+        <x:v>https://github.com/jackconnolly1000-ux/sec-filing-research-terminal/blob/main/docs/borrowing_lease_presentation.md</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add checked two-date company history
</commit_message>
<xml_diff>
--- a/samples/lly_liquidity.xlsx
+++ b/samples/lly_liquidity.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding conclusion" sheetId="1" r:id="R44ba2e92ab82474f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Borrowing and leases" sheetId="2" r:id="R42fc5e91854f41a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt and liquidity" sheetId="3" r:id="R559c9296e69743ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repayment review" sheetId="4" r:id="R7c8a89892f0c44b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="5" r:id="R6ce6e94b33334fc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="6" r:id="R8d2c326248f74d6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding conclusion" sheetId="1" r:id="R47119031e9e14377"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Borrowing and leases" sheetId="2" r:id="R1eadd7c12bda4566"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt and liquidity" sheetId="3" r:id="R00ee6960dee7402b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="History" sheetId="4" r:id="Rec05d0b4eb2448e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repayment review" sheetId="5" r:id="R08107539c00f443e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="6" r:id="Re4870f8b713940cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="7" r:id="R1de904192b7a4b79"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -372,7 +373,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="193">
+  <x:cellXfs count="221">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -889,6 +890,60 @@
     </x:xf>
     <x:xf numFmtId="201" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="13" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="13" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1087,7 +1142,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf65719a8d4ee4135"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R81d2be1fe1e74c04"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2370,6 +2425,259 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="43" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="29" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="29" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="85" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4"/>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="7" t="str">
+        <x:v>Eli Lilly and Company — dated history</x:v>
+      </x:c>
+      <x:c r="B2" s="4"/>
+      <x:c r="C2" s="4"/>
+      <x:c r="D2" s="4"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="8" t="str">
+        <x:v>USD millions unless x or %. Fiscal year and later TTM both span twelve months and overlap.</x:v>
+      </x:c>
+      <x:c r="B3" s="4"/>
+      <x:c r="C3" s="4"/>
+      <x:c r="D3" s="4"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="4"/>
+      <x:c r="B4" s="4"/>
+      <x:c r="C4" s="4"/>
+      <x:c r="D4" s="4"/>
+    </x:row>
+    <x:row r="5" ht="32" customHeight="1">
+      <x:c r="A5" s="13" t="str">
+        <x:v>Measure</x:v>
+      </x:c>
+      <x:c r="B5" s="96" t="str">
+        <x:v>As of / FY ended 2025-12-31</x:v>
+      </x:c>
+      <x:c r="C5" s="96" t="str">
+        <x:v>As of / TTM ended 2026-06-30</x:v>
+      </x:c>
+      <x:c r="D5" s="14" t="str">
+        <x:v>Basis / limits</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="45" customHeight="1">
+      <x:c r="A6" s="25" t="str">
+        <x:v>Cash and cash equivalents</x:v>
+      </x:c>
+      <x:c r="B6" s="125" t="n">
+        <x:f>IF(ISNUMBER('Data'!B130),'Data'!B130,NA())</x:f>
+        <x:v>7268000000</x:v>
+      </x:c>
+      <x:c r="C6" s="125" t="n">
+        <x:f>'Debt and liquidity'!B6</x:f>
+        <x:v>8950000000</x:v>
+      </x:c>
+      <x:c r="D6" s="16" t="str">
+        <x:v>Cash and cash equivalents excluding restricted cash. Investments are not substituted.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="62" customHeight="1">
+      <x:c r="A7" s="25" t="str">
+        <x:v>Baseline gross debt</x:v>
+      </x:c>
+      <x:c r="B7" s="125" t="n">
+        <x:f>IF(ISNUMBER('Data'!B133),'Data'!B133,NA())+IF(ISNUMBER('Data'!B134),'Data'!B134,NA())</x:f>
+        <x:v>42503000000</x:v>
+      </x:c>
+      <x:c r="C7" s="125" t="n">
+        <x:f>'Debt and liquidity'!B7</x:f>
+        <x:v>54908000000</x:v>
+      </x:c>
+      <x:c r="D7" s="16" t="str">
+        <x:v>Carrying amount of borrowing. Operating/finance leases and commitments are excluded. In this 10-Q, the Note 8 fair-value table's carrying amounts (commercial paper 5,284M plus long-term debt including current portion 49,624M) present the same 54,908M; they are not added.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="45" customHeight="1">
+      <x:c r="A8" s="25" t="str">
+        <x:v>Net debt</x:v>
+      </x:c>
+      <x:c r="B8" s="186" t="n">
+        <x:f>B7-B6</x:f>
+        <x:v>35235000000</x:v>
+      </x:c>
+      <x:c r="C8" s="125" t="n">
+        <x:f>'Debt and liquidity'!B8</x:f>
+        <x:v>45958000000</x:v>
+      </x:c>
+      <x:c r="D8" s="16" t="str">
+        <x:v>Baseline borrowing less cash excluding restricted cash. Same date and filing. Negative net debt is retained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="49" customHeight="1">
+      <x:c r="A9" s="25" t="str">
+        <x:v>Current ratio</x:v>
+      </x:c>
+      <x:c r="B9" s="162" t="n">
+        <x:f>IF(IF(ISNUMBER('Data'!B132),'Data'!B132,NA())&gt;0,IF(ISNUMBER('Data'!B131),'Data'!B131,NA())/IF(ISNUMBER('Data'!B132),'Data'!B132,NA()),NA())</x:f>
+        <x:v>1.5791132054047916</x:v>
+      </x:c>
+      <x:c r="C9" s="162" t="n">
+        <x:f>'Debt and liquidity'!B9</x:f>
+        <x:v>1.3546427598919168</x:v>
+      </x:c>
+      <x:c r="D9" s="16" t="str">
+        <x:v>Total current assets / total current liabilities from one balance sheet. Liabilities include more than borrowing; assets include more than cash.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="45" customHeight="1">
+      <x:c r="A10" s="25" t="str">
+        <x:v>Operating cash flow</x:v>
+      </x:c>
+      <x:c r="B10" s="125" t="n">
+        <x:f>IF(ISNUMBER('Data'!B135),'Data'!B135,NA())</x:f>
+        <x:v>16813000000</x:v>
+      </x:c>
+      <x:c r="C10" s="125" t="n">
+        <x:f>'Debt and liquidity'!B10</x:f>
+        <x:v>28083000000</x:v>
+      </x:c>
+      <x:c r="D10" s="16" t="str">
+        <x:v>Reported historical OCF; recurrence is not established. Uses FY + current YTD - prior YTD.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="45" customHeight="1">
+      <x:c r="A11" s="25" t="str">
+        <x:v>Purchases of property and equipment</x:v>
+      </x:c>
+      <x:c r="B11" s="125" t="n">
+        <x:f>IF(ISNUMBER('Data'!B136),'Data'!B136,NA())</x:f>
+        <x:v>7841000000</x:v>
+      </x:c>
+      <x:c r="C11" s="125" t="n">
+        <x:f>'Debt and liquidity'!B11</x:f>
+        <x:v>9893000000</x:v>
+      </x:c>
+      <x:c r="D11" s="16" t="str">
+        <x:v>Reported purchases of property and equipment; excludes acquisitions and other investing cash flows.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="45" customHeight="1">
+      <x:c r="A12" s="25" t="str">
+        <x:v>Free cash flow</x:v>
+      </x:c>
+      <x:c r="B12" s="186" t="n">
+        <x:f>B10-B11</x:f>
+        <x:v>8972000000</x:v>
+      </x:c>
+      <x:c r="C12" s="125" t="n">
+        <x:f>'Debt and liquidity'!B12</x:f>
+        <x:v>18190000000</x:v>
+      </x:c>
+      <x:c r="D12" s="16" t="str">
+        <x:v>OCF less reported capital spending. Uses the spending basis above; excludes acquisitions, dividends and other cash uses.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="45" customHeight="1">
+      <x:c r="A13" s="25" t="str">
+        <x:v>Operating cash flow / debt</x:v>
+      </x:c>
+      <x:c r="B13" s="163" t="n">
+        <x:f>IF(B7&gt;0,B10/B7,NA())</x:f>
+        <x:v>0.3955720772651342</x:v>
+      </x:c>
+      <x:c r="C13" s="216" t="n">
+        <x:f>'Debt and liquidity'!B13</x:f>
+        <x:v>0.511455525606469</x:v>
+      </x:c>
+      <x:c r="D13" s="16" t="str">
+        <x:v>Twelve-month OCF / borrowing at each period end. Prior column uses the fiscal year; later column uses TTM. Not repayment coverage.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="45" customHeight="1">
+      <x:c r="A14" s="25" t="str">
+        <x:v>Free cash flow / debt</x:v>
+      </x:c>
+      <x:c r="B14" s="163" t="n">
+        <x:f>IF(B7&gt;0,B12/B7,NA())</x:f>
+        <x:v>0.2110909818130485</x:v>
+      </x:c>
+      <x:c r="C14" s="216" t="n">
+        <x:f>'Debt and liquidity'!B14</x:f>
+        <x:v>0.33128141618707657</x:v>
+      </x:c>
+      <x:c r="D14" s="16" t="str">
+        <x:v>Twelve-month FCF / borrowing at each period end. Prior column uses the fiscal year; later column uses TTM. Not repayment coverage.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="88" customHeight="1">
+      <x:c r="A15" s="26" t="str">
+        <x:v>Historical interest coverage</x:v>
+      </x:c>
+      <x:c r="B15" s="217" t="n">
+        <x:f>IF(AND('Debt and liquidity'!B46&gt;0,'Debt and liquidity'!B44=0),'Debt and liquidity'!B40/'Debt and liquidity'!B46,NA())</x:f>
+        <x:v>29.387709497206703</x:v>
+      </x:c>
+      <x:c r="C15" s="217" t="n">
+        <x:f>'Debt and liquidity'!B15</x:f>
+        <x:v>31.17052826691381</x:v>
+      </x:c>
+      <x:c r="D15" s="18" t="str">
+        <x:v>FY2025 Note 11 explicitly reports interest on borrowings net of capitalized interest. The interim segment table labels the line interest expense without explicitly stating its capitalization basis. All three amounts are used as reported, before any interest-income offset. Capitalized interest is not added or subtracted; its amount and total interest incurred are Unavailable.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="4"/>
+      <x:c r="B16" s="4"/>
+      <x:c r="C16" s="4"/>
+      <x:c r="D16" s="4"/>
+    </x:row>
+    <x:row r="17" ht="70" customHeight="1">
+      <x:c r="A17" s="4" t="str">
+        <x:v>Period definitions</x:v>
+      </x:c>
+      <x:c r="B17" s="4"/>
+      <x:c r="C17" s="4"/>
+      <x:c r="D17" s="4" t="str">
+        <x:v>Balance-sheet figures compare the stated dates. Flows and interest coverage compare a fiscal year with a later TTM: both span twelve months and overlap. No interim annualization, independent-period growth rate or future repayment coverage is inferred.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="4" t="str">
+        <x:v>Fiscal-year flows</x:v>
+      </x:c>
+      <x:c r="B18" s="4"/>
+      <x:c r="C18" s="4"/>
+      <x:c r="D18" s="4" t="str">
+        <x:v>2025-01-01 to 2025-12-31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="4" t="str">
+        <x:v>Later TTM flows</x:v>
+      </x:c>
+      <x:c r="B19" s="4"/>
+      <x:c r="C19" s="4"/>
+      <x:c r="D19" s="4" t="str">
+        <x:v>2025-07-01 to 2026-06-30</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="46" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
@@ -3952,11 +4260,11 @@
     <x:mergeCell ref="A96:D96"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7fa7867d1754332"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1ec28f33921480d"/>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -9805,12 +10113,360 @@
       </x:c>
       <x:c r="O126" s="18" t="str"/>
     </x:row>
+    <x:row r="129" ht="70" customHeight="1">
+      <x:c r="A129" s="13" t="str">
+        <x:v>Input</x:v>
+      </x:c>
+      <x:c r="B129" s="96" t="str">
+        <x:v>USD millions</x:v>
+      </x:c>
+      <x:c r="C129" s="96" t="str">
+        <x:v>Period start</x:v>
+      </x:c>
+      <x:c r="D129" s="96" t="str">
+        <x:v>Period end</x:v>
+      </x:c>
+      <x:c r="E129" s="96" t="str">
+        <x:v>Form</x:v>
+      </x:c>
+      <x:c r="F129" s="96" t="str">
+        <x:v>Filed</x:v>
+      </x:c>
+      <x:c r="G129" s="96" t="str">
+        <x:v>Accession</x:v>
+      </x:c>
+      <x:c r="H129" s="96" t="str">
+        <x:v>Tag</x:v>
+      </x:c>
+      <x:c r="I129" s="96" t="str">
+        <x:v>Context</x:v>
+      </x:c>
+      <x:c r="J129" s="96" t="str">
+        <x:v>Scale</x:v>
+      </x:c>
+      <x:c r="K129" s="96" t="str">
+        <x:v>Decimals</x:v>
+      </x:c>
+      <x:c r="L129" s="96" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="M129" s="96" t="str">
+        <x:v>Selection rule</x:v>
+      </x:c>
+      <x:c r="N129" s="96" t="str">
+        <x:v>Unavailable reason</x:v>
+      </x:c>
+      <x:c r="O129" s="14" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130" ht="70" customHeight="1">
+      <x:c r="A130" s="25" t="str">
+        <x:v>Cash and cash equivalents</x:v>
+      </x:c>
+      <x:c r="B130" s="106" t="n">
+        <x:v>7268000000</x:v>
+      </x:c>
+      <x:c r="C130" s="76"/>
+      <x:c r="D130" s="76" t="d">
+        <x:v>2025-12-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E130" s="107" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F130" s="76" t="d">
+        <x:v>2026-02-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G130" s="107" t="str">
+        <x:v>0000059478-26-000013</x:v>
+      </x:c>
+      <x:c r="H130" s="107" t="str">
+        <x:v>us-gaap:CashAndCashEquivalentsAtCarryingValue</x:v>
+      </x:c>
+      <x:c r="I130" s="107" t="str">
+        <x:v>c-16</x:v>
+      </x:c>
+      <x:c r="J130" s="107" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K130" s="107" t="str">
+        <x:v>-6</x:v>
+      </x:c>
+      <x:c r="L130" s="107" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/59478/000005947826000013/lly-20251231.htm</x:v>
+      </x:c>
+      <x:c r="M130" s="107" t="str">
+        <x:v>10-K balance sheet p. 56; cash flows p. 58</x:v>
+      </x:c>
+      <x:c r="N130" s="107" t="str"/>
+      <x:c r="O130" s="16" t="str">
+        <x:v>d45f8d1e0945df0b7b30254e96ff8c5dbd1df7d15b17c8ef7399c8e0206b7d7f</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="70" customHeight="1">
+      <x:c r="A131" s="25" t="str">
+        <x:v>Current assets</x:v>
+      </x:c>
+      <x:c r="B131" s="106" t="n">
+        <x:v>55629000000</x:v>
+      </x:c>
+      <x:c r="C131" s="76"/>
+      <x:c r="D131" s="76" t="d">
+        <x:v>2025-12-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E131" s="107" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F131" s="76" t="d">
+        <x:v>2026-02-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G131" s="107" t="str">
+        <x:v>0000059478-26-000013</x:v>
+      </x:c>
+      <x:c r="H131" s="107" t="str">
+        <x:v>us-gaap:AssetsCurrent</x:v>
+      </x:c>
+      <x:c r="I131" s="107" t="str">
+        <x:v>c-16</x:v>
+      </x:c>
+      <x:c r="J131" s="107" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K131" s="107" t="str">
+        <x:v>-6</x:v>
+      </x:c>
+      <x:c r="L131" s="107" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/59478/000005947826000013/lly-20251231.htm</x:v>
+      </x:c>
+      <x:c r="M131" s="107" t="str">
+        <x:v>10-K balance sheet p. 56; cash flows p. 58</x:v>
+      </x:c>
+      <x:c r="N131" s="107" t="str"/>
+      <x:c r="O131" s="16" t="str">
+        <x:v>d45f8d1e0945df0b7b30254e96ff8c5dbd1df7d15b17c8ef7399c8e0206b7d7f</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132" ht="70" customHeight="1">
+      <x:c r="A132" s="25" t="str">
+        <x:v>Current liabilities</x:v>
+      </x:c>
+      <x:c r="B132" s="106" t="n">
+        <x:v>35228000000</x:v>
+      </x:c>
+      <x:c r="C132" s="76"/>
+      <x:c r="D132" s="76" t="d">
+        <x:v>2025-12-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E132" s="107" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F132" s="76" t="d">
+        <x:v>2026-02-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G132" s="107" t="str">
+        <x:v>0000059478-26-000013</x:v>
+      </x:c>
+      <x:c r="H132" s="107" t="str">
+        <x:v>us-gaap:LiabilitiesCurrent</x:v>
+      </x:c>
+      <x:c r="I132" s="107" t="str">
+        <x:v>c-16</x:v>
+      </x:c>
+      <x:c r="J132" s="107" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K132" s="107" t="str">
+        <x:v>-6</x:v>
+      </x:c>
+      <x:c r="L132" s="107" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/59478/000005947826000013/lly-20251231.htm</x:v>
+      </x:c>
+      <x:c r="M132" s="107" t="str">
+        <x:v>10-K balance sheet p. 56; cash flows p. 58</x:v>
+      </x:c>
+      <x:c r="N132" s="107" t="str"/>
+      <x:c r="O132" s="16" t="str">
+        <x:v>d45f8d1e0945df0b7b30254e96ff8c5dbd1df7d15b17c8ef7399c8e0206b7d7f</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" ht="70" customHeight="1">
+      <x:c r="A133" s="25" t="str">
+        <x:v>Short-term borrowings and current maturities of long-term debt</x:v>
+      </x:c>
+      <x:c r="B133" s="106" t="n">
+        <x:v>1635000000</x:v>
+      </x:c>
+      <x:c r="C133" s="76"/>
+      <x:c r="D133" s="76" t="d">
+        <x:v>2025-12-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E133" s="107" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F133" s="76" t="d">
+        <x:v>2026-02-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G133" s="107" t="str">
+        <x:v>0000059478-26-000013</x:v>
+      </x:c>
+      <x:c r="H133" s="107" t="str">
+        <x:v>us-gaap:DebtCurrent</x:v>
+      </x:c>
+      <x:c r="I133" s="107" t="str">
+        <x:v>c-16</x:v>
+      </x:c>
+      <x:c r="J133" s="107" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K133" s="107" t="str">
+        <x:v>-6</x:v>
+      </x:c>
+      <x:c r="L133" s="107" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/59478/000005947826000013/lly-20251231.htm</x:v>
+      </x:c>
+      <x:c r="M133" s="107" t="str">
+        <x:v>10-K balance sheet p. 56; cash flows p. 58</x:v>
+      </x:c>
+      <x:c r="N133" s="107" t="str"/>
+      <x:c r="O133" s="16" t="str">
+        <x:v>d45f8d1e0945df0b7b30254e96ff8c5dbd1df7d15b17c8ef7399c8e0206b7d7f</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134" ht="70" customHeight="1">
+      <x:c r="A134" s="25" t="str">
+        <x:v>Long-term debt</x:v>
+      </x:c>
+      <x:c r="B134" s="106" t="n">
+        <x:v>40868000000</x:v>
+      </x:c>
+      <x:c r="C134" s="76"/>
+      <x:c r="D134" s="76" t="d">
+        <x:v>2025-12-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E134" s="107" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F134" s="76" t="d">
+        <x:v>2026-02-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G134" s="107" t="str">
+        <x:v>0000059478-26-000013</x:v>
+      </x:c>
+      <x:c r="H134" s="107" t="str">
+        <x:v>us-gaap:LongTermDebtNoncurrent</x:v>
+      </x:c>
+      <x:c r="I134" s="107" t="str">
+        <x:v>c-16</x:v>
+      </x:c>
+      <x:c r="J134" s="107" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K134" s="107" t="str">
+        <x:v>-6</x:v>
+      </x:c>
+      <x:c r="L134" s="107" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/59478/000005947826000013/lly-20251231.htm</x:v>
+      </x:c>
+      <x:c r="M134" s="107" t="str">
+        <x:v>10-K balance sheet p. 56; cash flows p. 58</x:v>
+      </x:c>
+      <x:c r="N134" s="107" t="str"/>
+      <x:c r="O134" s="16" t="str">
+        <x:v>d45f8d1e0945df0b7b30254e96ff8c5dbd1df7d15b17c8ef7399c8e0206b7d7f</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135" ht="70" customHeight="1">
+      <x:c r="A135" s="25" t="str">
+        <x:v>Operating cash flow · fiscal year</x:v>
+      </x:c>
+      <x:c r="B135" s="106" t="n">
+        <x:v>16813000000</x:v>
+      </x:c>
+      <x:c r="C135" s="76" t="d">
+        <x:v>2025-01-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D135" s="76" t="d">
+        <x:v>2025-12-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E135" s="107" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F135" s="76" t="d">
+        <x:v>2026-02-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G135" s="107" t="str">
+        <x:v>0000059478-26-000013</x:v>
+      </x:c>
+      <x:c r="H135" s="107" t="str">
+        <x:v>us-gaap:NetCashProvidedByUsedInOperatingActivities</x:v>
+      </x:c>
+      <x:c r="I135" s="107" t="str">
+        <x:v>c-1</x:v>
+      </x:c>
+      <x:c r="J135" s="107" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K135" s="107" t="str">
+        <x:v>-6</x:v>
+      </x:c>
+      <x:c r="L135" s="107" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/59478/000005947826000013/lly-20251231.htm</x:v>
+      </x:c>
+      <x:c r="M135" s="107" t="str">
+        <x:v>Annual cash-flow statement</x:v>
+      </x:c>
+      <x:c r="N135" s="107" t="str"/>
+      <x:c r="O135" s="16" t="str"/>
+    </x:row>
+    <x:row r="136" ht="70" customHeight="1">
+      <x:c r="A136" s="26" t="str">
+        <x:v>Purchases of property and equipment · fiscal year</x:v>
+      </x:c>
+      <x:c r="B136" s="108" t="n">
+        <x:v>7841000000</x:v>
+      </x:c>
+      <x:c r="C136" s="80" t="d">
+        <x:v>2025-01-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D136" s="80" t="d">
+        <x:v>2025-12-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E136" s="109" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="F136" s="80" t="d">
+        <x:v>2026-02-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G136" s="109" t="str">
+        <x:v>0000059478-26-000013</x:v>
+      </x:c>
+      <x:c r="H136" s="109" t="str">
+        <x:v>us-gaap:PaymentsToAcquireOtherPropertyPlantAndEquipment</x:v>
+      </x:c>
+      <x:c r="I136" s="109" t="str">
+        <x:v>c-1</x:v>
+      </x:c>
+      <x:c r="J136" s="109" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K136" s="109" t="str">
+        <x:v>-6</x:v>
+      </x:c>
+      <x:c r="L136" s="109" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/59478/000005947826000013/lly-20251231.htm</x:v>
+      </x:c>
+      <x:c r="M136" s="109" t="str">
+        <x:v>Annual cash-flow statement</x:v>
+      </x:c>
+      <x:c r="N136" s="109" t="str"/>
+      <x:c r="O136" s="18" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -9971,6 +10627,17 @@
         <x:v>https://github.com/jackconnolly1000-ux/sec-filing-research-terminal/blob/main/docs/borrowing_lease_presentation.md</x:v>
       </x:c>
     </x:row>
+    <x:row r="15" ht="70" customHeight="1">
+      <x:c r="A15" s="218" t="str">
+        <x:v>History</x:v>
+      </x:c>
+      <x:c r="B15" s="219" t="str">
+        <x:v>Two dated observations per company. Fiscal-year and TTM flows are overlapping twelve-month windows. Unsupported older Vistra borrowing and dependent ratios remain Unavailable.</x:v>
+      </x:c>
+      <x:c r="C15" s="220" t="str">
+        <x:v>https://github.com/jackconnolly1000-ux/sec-filing-research-terminal/blob/main/docs/company_history.md</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add two checked chart questions to company reviews and exports
</commit_message>
<xml_diff>
--- a/samples/lly_liquidity.xlsx
+++ b/samples/lly_liquidity.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding conclusion" sheetId="1" r:id="R47119031e9e14377"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Borrowing and leases" sheetId="2" r:id="R1eadd7c12bda4566"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt and liquidity" sheetId="3" r:id="R00ee6960dee7402b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="History" sheetId="4" r:id="Rec05d0b4eb2448e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repayment review" sheetId="5" r:id="R08107539c00f443e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="6" r:id="Re4870f8b713940cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="7" r:id="R1de904192b7a4b79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding conclusion" sheetId="1" r:id="R545cd74760084c87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Borrowing and leases" sheetId="2" r:id="R238cedd23ec247d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt and liquidity" sheetId="3" r:id="Rd81cc1e44b5f4b44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="History" sheetId="4" r:id="R36028c37b97841dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core charts" sheetId="5" r:id="Ra3a09e8001d84070"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repayment review" sheetId="6" r:id="Rf3d8710805a74af5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="7" r:id="R1a331d15f7f4430c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="8" r:id="R32f8516f62b34357"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -373,7 +374,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="221">
+  <x:cellXfs count="222">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -945,6 +946,9 @@
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="13" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -953,6 +957,418 @@
 </file>
 
 <file path=xl/drawings/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:rPr sz="900">
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:rPr>
+              <a:t>What remained after capital spending?</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="900">
+              <a:latin typeface="Arial"/>
+              <a:ea typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>USD millions</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="8D99A8"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Core charts'!$A$6:$A$8</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Core charts'!$B$6:$B$8</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0,,;(#,##0,,);"-"</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="750">
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48672768"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:r>
+                  <a:t>USD millions</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="#,##0,,;(#,##0,,)" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="750">
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr>
+              <a:latin typeface="Arial"/>
+              <a:ea typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:rPr sz="900">
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:rPr>
+              <a:t>How did borrowing and cash change?</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="900">
+              <a:latin typeface="Arial"/>
+              <a:ea typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Cash and equivalents</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="8D99A8"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Core charts'!$A$25:$A$26</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Core charts'!$B$25:$B$26</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0,,;(#,##0,,);"-"</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Baseline borrowing</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="47627F"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Core charts'!$A$25:$A$26</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Core charts'!$C$25:$C$26</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0,,;(#,##0,,);"-"</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="750">
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48672768"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:r>
+                  <a:t>USD millions</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="#,##0,,;(#,##0,,)" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="750">
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr>
+              <a:latin typeface="Arial"/>
+              <a:ea typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -1122,6 +1538,71 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8ebdb1b61a44431d"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5d1e072ed27a4814"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
@@ -1142,7 +1623,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R81d2be1fe1e74c04"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb8fd9f5b2b7b470e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2678,6 +3159,817 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="3" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="10" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="10" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="10" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="10" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="10" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="10" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="10" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="10" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="10" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="10" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="35" customHeight="1">
+      <x:c r="A1" s="4"/>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
+      <x:c r="G1" s="2"/>
+      <x:c r="H1" s="2"/>
+      <x:c r="I1" s="2"/>
+      <x:c r="J1" s="2"/>
+      <x:c r="K1" s="2"/>
+      <x:c r="L1" s="2"/>
+      <x:c r="M1" s="2"/>
+      <x:c r="N1" s="2"/>
+      <x:c r="O1" s="2"/>
+    </x:row>
+    <x:row r="2" ht="35" customHeight="1">
+      <x:c r="A2" s="7" t="str">
+        <x:v>LLY — two chart questions</x:v>
+      </x:c>
+      <x:c r="B2" s="4"/>
+      <x:c r="C2" s="4"/>
+      <x:c r="D2" s="4"/>
+      <x:c r="E2" s="2"/>
+      <x:c r="F2" s="2"/>
+      <x:c r="G2" s="2"/>
+      <x:c r="H2" s="2"/>
+      <x:c r="I2" s="2"/>
+      <x:c r="J2" s="2"/>
+      <x:c r="K2" s="2"/>
+      <x:c r="L2" s="2"/>
+      <x:c r="M2" s="2"/>
+      <x:c r="N2" s="2"/>
+      <x:c r="O2" s="2"/>
+    </x:row>
+    <x:row r="3" ht="35" customHeight="1">
+      <x:c r="A3" s="8" t="str">
+        <x:v>TTM 2025-07-01 to 2026-06-30. Values stored in USD, displayed in millions.</x:v>
+      </x:c>
+      <x:c r="B3" s="4"/>
+      <x:c r="C3" s="4"/>
+      <x:c r="D3" s="4"/>
+      <x:c r="E3" s="2"/>
+      <x:c r="F3" s="2"/>
+      <x:c r="G3" s="2"/>
+      <x:c r="H3" s="2"/>
+      <x:c r="I3" s="2"/>
+      <x:c r="J3" s="2"/>
+      <x:c r="K3" s="2"/>
+      <x:c r="L3" s="2"/>
+      <x:c r="M3" s="2"/>
+      <x:c r="N3" s="2"/>
+      <x:c r="O3" s="2"/>
+    </x:row>
+    <x:row r="4" ht="35" customHeight="1">
+      <x:c r="A4" s="4"/>
+      <x:c r="B4" s="4"/>
+      <x:c r="C4" s="4"/>
+      <x:c r="D4" s="4"/>
+      <x:c r="E4" s="2"/>
+      <x:c r="F4" s="2"/>
+      <x:c r="G4" s="2"/>
+      <x:c r="H4" s="2"/>
+      <x:c r="I4" s="2"/>
+      <x:c r="J4" s="2"/>
+      <x:c r="K4" s="2"/>
+      <x:c r="L4" s="2"/>
+      <x:c r="M4" s="2"/>
+      <x:c r="N4" s="2"/>
+      <x:c r="O4" s="2"/>
+    </x:row>
+    <x:row r="5" ht="35" customHeight="1">
+      <x:c r="A5" s="13" t="str">
+        <x:v>TTM measure</x:v>
+      </x:c>
+      <x:c r="B5" s="14" t="str">
+        <x:v>USD millions</x:v>
+      </x:c>
+      <x:c r="C5" s="4"/>
+      <x:c r="D5" s="4"/>
+      <x:c r="E5" s="2"/>
+      <x:c r="F5" s="2"/>
+      <x:c r="G5" s="2"/>
+      <x:c r="H5" s="2"/>
+      <x:c r="I5" s="2"/>
+      <x:c r="J5" s="2"/>
+      <x:c r="K5" s="2"/>
+      <x:c r="L5" s="2"/>
+      <x:c r="M5" s="2"/>
+      <x:c r="N5" s="2"/>
+      <x:c r="O5" s="2"/>
+    </x:row>
+    <x:row r="6" ht="35" customHeight="1">
+      <x:c r="A6" s="25" t="str">
+        <x:v>Operating cash flow</x:v>
+      </x:c>
+      <x:c r="B6" s="144" t="n">
+        <x:f>'Debt and liquidity'!B10</x:f>
+        <x:v>28083000000</x:v>
+      </x:c>
+      <x:c r="C6" s="4"/>
+      <x:c r="D6" s="4"/>
+      <x:c r="E6" s="2"/>
+      <x:c r="F6" s="2"/>
+      <x:c r="G6" s="2"/>
+      <x:c r="H6" s="2"/>
+      <x:c r="I6" s="2"/>
+      <x:c r="J6" s="2"/>
+      <x:c r="K6" s="2"/>
+      <x:c r="L6" s="2"/>
+      <x:c r="M6" s="2"/>
+      <x:c r="N6" s="2"/>
+      <x:c r="O6" s="2"/>
+    </x:row>
+    <x:row r="7" ht="35" customHeight="1">
+      <x:c r="A7" s="25" t="str">
+        <x:v>Capital spending</x:v>
+      </x:c>
+      <x:c r="B7" s="144" t="n">
+        <x:f>-'Debt and liquidity'!B11</x:f>
+        <x:v>-9893000000</x:v>
+      </x:c>
+      <x:c r="C7" s="4"/>
+      <x:c r="D7" s="4"/>
+      <x:c r="E7" s="2"/>
+      <x:c r="F7" s="2"/>
+      <x:c r="G7" s="2"/>
+      <x:c r="H7" s="2"/>
+      <x:c r="I7" s="2"/>
+      <x:c r="J7" s="2"/>
+      <x:c r="K7" s="2"/>
+      <x:c r="L7" s="2"/>
+      <x:c r="M7" s="2"/>
+      <x:c r="N7" s="2"/>
+      <x:c r="O7" s="2"/>
+    </x:row>
+    <x:row r="8" ht="35" customHeight="1">
+      <x:c r="A8" s="26" t="str">
+        <x:v>Free cash flow</x:v>
+      </x:c>
+      <x:c r="B8" s="221" t="n">
+        <x:f>'Debt and liquidity'!B12</x:f>
+        <x:v>18190000000</x:v>
+      </x:c>
+      <x:c r="C8" s="4"/>
+      <x:c r="D8" s="4"/>
+      <x:c r="E8" s="2"/>
+      <x:c r="F8" s="2"/>
+      <x:c r="G8" s="2"/>
+      <x:c r="H8" s="2"/>
+      <x:c r="I8" s="2"/>
+      <x:c r="J8" s="2"/>
+      <x:c r="K8" s="2"/>
+      <x:c r="L8" s="2"/>
+      <x:c r="M8" s="2"/>
+      <x:c r="N8" s="2"/>
+      <x:c r="O8" s="2"/>
+    </x:row>
+    <x:row r="9" ht="35" customHeight="1">
+      <x:c r="A9" s="4"/>
+      <x:c r="B9" s="4"/>
+      <x:c r="C9" s="4"/>
+      <x:c r="D9" s="4"/>
+      <x:c r="E9" s="2"/>
+      <x:c r="F9" s="2"/>
+      <x:c r="G9" s="2"/>
+      <x:c r="H9" s="2"/>
+      <x:c r="I9" s="2"/>
+      <x:c r="J9" s="2"/>
+      <x:c r="K9" s="2"/>
+      <x:c r="L9" s="2"/>
+      <x:c r="M9" s="2"/>
+      <x:c r="N9" s="2"/>
+      <x:c r="O9" s="2"/>
+    </x:row>
+    <x:row r="10" ht="80" customHeight="1">
+      <x:c r="A10" s="4" t="str">
+        <x:v>Calculation basis</x:v>
+      </x:c>
+      <x:c r="B10" s="4"/>
+      <x:c r="C10" s="4"/>
+      <x:c r="D10" s="4" t="str">
+        <x:v>FCF = OCF − capital spending. FCF is a result, not an additional cash flow. Capital spending is shown negative.</x:v>
+      </x:c>
+      <x:c r="E10" s="2"/>
+      <x:c r="F10" s="2"/>
+      <x:c r="G10" s="2"/>
+      <x:c r="H10" s="2"/>
+      <x:c r="I10" s="2"/>
+      <x:c r="J10" s="2"/>
+      <x:c r="K10" s="2"/>
+      <x:c r="L10" s="2"/>
+      <x:c r="M10" s="2"/>
+      <x:c r="N10" s="2"/>
+      <x:c r="O10" s="2"/>
+    </x:row>
+    <x:row r="11" ht="35" customHeight="1">
+      <x:c r="A11" s="4"/>
+      <x:c r="B11" s="4"/>
+      <x:c r="C11" s="4"/>
+      <x:c r="D11" s="4"/>
+      <x:c r="E11" s="2"/>
+      <x:c r="F11" s="2"/>
+      <x:c r="G11" s="2"/>
+      <x:c r="H11" s="2"/>
+      <x:c r="I11" s="2"/>
+      <x:c r="J11" s="2"/>
+      <x:c r="K11" s="2"/>
+      <x:c r="L11" s="2"/>
+      <x:c r="M11" s="2"/>
+      <x:c r="N11" s="2"/>
+      <x:c r="O11" s="2"/>
+    </x:row>
+    <x:row r="12" ht="35" customHeight="1">
+      <x:c r="A12" s="4"/>
+      <x:c r="B12" s="4"/>
+      <x:c r="C12" s="4"/>
+      <x:c r="D12" s="4"/>
+      <x:c r="E12" s="2"/>
+      <x:c r="F12" s="2"/>
+      <x:c r="G12" s="2"/>
+      <x:c r="H12" s="2"/>
+      <x:c r="I12" s="2"/>
+      <x:c r="J12" s="2"/>
+      <x:c r="K12" s="2"/>
+      <x:c r="L12" s="2"/>
+      <x:c r="M12" s="2"/>
+      <x:c r="N12" s="2"/>
+      <x:c r="O12" s="2"/>
+    </x:row>
+    <x:row r="13" ht="35" customHeight="1">
+      <x:c r="A13" s="4"/>
+      <x:c r="B13" s="4"/>
+      <x:c r="C13" s="4"/>
+      <x:c r="D13" s="4"/>
+      <x:c r="E13" s="2"/>
+      <x:c r="F13" s="2"/>
+      <x:c r="G13" s="2"/>
+      <x:c r="H13" s="2"/>
+      <x:c r="I13" s="2"/>
+      <x:c r="J13" s="2"/>
+      <x:c r="K13" s="2"/>
+      <x:c r="L13" s="2"/>
+      <x:c r="M13" s="2"/>
+      <x:c r="N13" s="2"/>
+      <x:c r="O13" s="2"/>
+    </x:row>
+    <x:row r="14" ht="35" customHeight="1">
+      <x:c r="A14" s="4"/>
+      <x:c r="B14" s="4"/>
+      <x:c r="C14" s="4"/>
+      <x:c r="D14" s="4"/>
+      <x:c r="E14" s="2"/>
+      <x:c r="F14" s="2"/>
+      <x:c r="G14" s="2"/>
+      <x:c r="H14" s="2"/>
+      <x:c r="I14" s="2"/>
+      <x:c r="J14" s="2"/>
+      <x:c r="K14" s="2"/>
+      <x:c r="L14" s="2"/>
+      <x:c r="M14" s="2"/>
+      <x:c r="N14" s="2"/>
+      <x:c r="O14" s="2"/>
+    </x:row>
+    <x:row r="15" ht="35" customHeight="1">
+      <x:c r="A15" s="4"/>
+      <x:c r="B15" s="4"/>
+      <x:c r="C15" s="4"/>
+      <x:c r="D15" s="4"/>
+      <x:c r="E15" s="2"/>
+      <x:c r="F15" s="2"/>
+      <x:c r="G15" s="2"/>
+      <x:c r="H15" s="2"/>
+      <x:c r="I15" s="2"/>
+      <x:c r="J15" s="2"/>
+      <x:c r="K15" s="2"/>
+      <x:c r="L15" s="2"/>
+      <x:c r="M15" s="2"/>
+      <x:c r="N15" s="2"/>
+      <x:c r="O15" s="2"/>
+    </x:row>
+    <x:row r="16" ht="35" customHeight="1">
+      <x:c r="A16" s="4"/>
+      <x:c r="B16" s="4"/>
+      <x:c r="C16" s="4"/>
+      <x:c r="D16" s="4"/>
+      <x:c r="E16" s="2"/>
+      <x:c r="F16" s="2"/>
+      <x:c r="G16" s="2"/>
+      <x:c r="H16" s="2"/>
+      <x:c r="I16" s="2"/>
+      <x:c r="J16" s="2"/>
+      <x:c r="K16" s="2"/>
+      <x:c r="L16" s="2"/>
+      <x:c r="M16" s="2"/>
+      <x:c r="N16" s="2"/>
+      <x:c r="O16" s="2"/>
+    </x:row>
+    <x:row r="17" ht="35" customHeight="1">
+      <x:c r="A17" s="4"/>
+      <x:c r="B17" s="4"/>
+      <x:c r="C17" s="4"/>
+      <x:c r="D17" s="4"/>
+      <x:c r="E17" s="2"/>
+      <x:c r="F17" s="2"/>
+      <x:c r="G17" s="2"/>
+      <x:c r="H17" s="2"/>
+      <x:c r="I17" s="2"/>
+      <x:c r="J17" s="2"/>
+      <x:c r="K17" s="2"/>
+      <x:c r="L17" s="2"/>
+      <x:c r="M17" s="2"/>
+      <x:c r="N17" s="2"/>
+      <x:c r="O17" s="2"/>
+    </x:row>
+    <x:row r="18" ht="35" customHeight="1">
+      <x:c r="A18" s="4"/>
+      <x:c r="B18" s="4"/>
+      <x:c r="C18" s="4"/>
+      <x:c r="D18" s="4"/>
+      <x:c r="E18" s="2"/>
+      <x:c r="F18" s="2"/>
+      <x:c r="G18" s="2"/>
+      <x:c r="H18" s="2"/>
+      <x:c r="I18" s="2"/>
+      <x:c r="J18" s="2"/>
+      <x:c r="K18" s="2"/>
+      <x:c r="L18" s="2"/>
+      <x:c r="M18" s="2"/>
+      <x:c r="N18" s="2"/>
+      <x:c r="O18" s="2"/>
+    </x:row>
+    <x:row r="19" ht="35" customHeight="1">
+      <x:c r="A19" s="4"/>
+      <x:c r="B19" s="4"/>
+      <x:c r="C19" s="4"/>
+      <x:c r="D19" s="4"/>
+      <x:c r="E19" s="2"/>
+      <x:c r="F19" s="2"/>
+      <x:c r="G19" s="2"/>
+      <x:c r="H19" s="2"/>
+      <x:c r="I19" s="2"/>
+      <x:c r="J19" s="2"/>
+      <x:c r="K19" s="2"/>
+      <x:c r="L19" s="2"/>
+      <x:c r="M19" s="2"/>
+      <x:c r="N19" s="2"/>
+      <x:c r="O19" s="2"/>
+    </x:row>
+    <x:row r="20" ht="35" customHeight="1">
+      <x:c r="A20" s="4"/>
+      <x:c r="B20" s="4"/>
+      <x:c r="C20" s="4"/>
+      <x:c r="D20" s="4"/>
+      <x:c r="E20" s="2"/>
+      <x:c r="F20" s="2"/>
+      <x:c r="G20" s="2"/>
+      <x:c r="H20" s="2"/>
+      <x:c r="I20" s="2"/>
+      <x:c r="J20" s="2"/>
+      <x:c r="K20" s="2"/>
+      <x:c r="L20" s="2"/>
+      <x:c r="M20" s="2"/>
+      <x:c r="N20" s="2"/>
+      <x:c r="O20" s="2"/>
+    </x:row>
+    <x:row r="21" ht="35" customHeight="1">
+      <x:c r="A21" s="4"/>
+      <x:c r="B21" s="4"/>
+      <x:c r="C21" s="4"/>
+      <x:c r="D21" s="4"/>
+      <x:c r="E21" s="2"/>
+      <x:c r="F21" s="2"/>
+      <x:c r="G21" s="2"/>
+      <x:c r="H21" s="2"/>
+      <x:c r="I21" s="2"/>
+      <x:c r="J21" s="2"/>
+      <x:c r="K21" s="2"/>
+      <x:c r="L21" s="2"/>
+      <x:c r="M21" s="2"/>
+      <x:c r="N21" s="2"/>
+      <x:c r="O21" s="2"/>
+    </x:row>
+    <x:row r="22" ht="35" customHeight="1">
+      <x:c r="A22" s="4"/>
+      <x:c r="B22" s="4"/>
+      <x:c r="C22" s="4"/>
+      <x:c r="D22" s="4"/>
+      <x:c r="E22" s="2"/>
+      <x:c r="F22" s="2"/>
+      <x:c r="G22" s="2"/>
+      <x:c r="H22" s="2"/>
+      <x:c r="I22" s="2"/>
+      <x:c r="J22" s="2"/>
+      <x:c r="K22" s="2"/>
+      <x:c r="L22" s="2"/>
+      <x:c r="M22" s="2"/>
+      <x:c r="N22" s="2"/>
+      <x:c r="O22" s="2"/>
+    </x:row>
+    <x:row r="23" ht="35" customHeight="1">
+      <x:c r="A23" s="4"/>
+      <x:c r="B23" s="4"/>
+      <x:c r="C23" s="4"/>
+      <x:c r="D23" s="4"/>
+      <x:c r="E23" s="2"/>
+      <x:c r="F23" s="2"/>
+      <x:c r="G23" s="2"/>
+      <x:c r="H23" s="2"/>
+      <x:c r="I23" s="2"/>
+      <x:c r="J23" s="2"/>
+      <x:c r="K23" s="2"/>
+      <x:c r="L23" s="2"/>
+      <x:c r="M23" s="2"/>
+      <x:c r="N23" s="2"/>
+      <x:c r="O23" s="2"/>
+    </x:row>
+    <x:row r="24" ht="35" customHeight="1">
+      <x:c r="A24" s="13" t="str">
+        <x:v>Balance-sheet date</x:v>
+      </x:c>
+      <x:c r="B24" s="96" t="str">
+        <x:v>Cash and equivalents</x:v>
+      </x:c>
+      <x:c r="C24" s="14" t="str">
+        <x:v>Baseline borrowing</x:v>
+      </x:c>
+      <x:c r="D24" s="4"/>
+      <x:c r="E24" s="2"/>
+      <x:c r="F24" s="2"/>
+      <x:c r="G24" s="2"/>
+      <x:c r="H24" s="2"/>
+      <x:c r="I24" s="2"/>
+      <x:c r="J24" s="2"/>
+      <x:c r="K24" s="2"/>
+      <x:c r="L24" s="2"/>
+      <x:c r="M24" s="2"/>
+      <x:c r="N24" s="2"/>
+      <x:c r="O24" s="2"/>
+    </x:row>
+    <x:row r="25" ht="35" customHeight="1">
+      <x:c r="A25" s="25" t="str">
+        <x:v>2025-12-31</x:v>
+      </x:c>
+      <x:c r="B25" s="125" t="n">
+        <x:f>'History'!B6</x:f>
+        <x:v>7268000000</x:v>
+      </x:c>
+      <x:c r="C25" s="144" t="n">
+        <x:f>'History'!B7</x:f>
+        <x:v>42503000000</x:v>
+      </x:c>
+      <x:c r="D25" s="4"/>
+      <x:c r="E25" s="2"/>
+      <x:c r="F25" s="2"/>
+      <x:c r="G25" s="2"/>
+      <x:c r="H25" s="2"/>
+      <x:c r="I25" s="2"/>
+      <x:c r="J25" s="2"/>
+      <x:c r="K25" s="2"/>
+      <x:c r="L25" s="2"/>
+      <x:c r="M25" s="2"/>
+      <x:c r="N25" s="2"/>
+      <x:c r="O25" s="2"/>
+    </x:row>
+    <x:row r="26" ht="35" customHeight="1">
+      <x:c r="A26" s="26" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="B26" s="129" t="n">
+        <x:f>'History'!C6</x:f>
+        <x:v>8950000000</x:v>
+      </x:c>
+      <x:c r="C26" s="221" t="n">
+        <x:f>'History'!C7</x:f>
+        <x:v>54908000000</x:v>
+      </x:c>
+      <x:c r="D26" s="4"/>
+      <x:c r="E26" s="2"/>
+      <x:c r="F26" s="2"/>
+      <x:c r="G26" s="2"/>
+      <x:c r="H26" s="2"/>
+      <x:c r="I26" s="2"/>
+      <x:c r="J26" s="2"/>
+      <x:c r="K26" s="2"/>
+      <x:c r="L26" s="2"/>
+      <x:c r="M26" s="2"/>
+      <x:c r="N26" s="2"/>
+      <x:c r="O26" s="2"/>
+    </x:row>
+    <x:row r="27" ht="35" customHeight="1">
+      <x:c r="A27" s="4"/>
+      <x:c r="B27" s="4"/>
+      <x:c r="C27" s="4"/>
+      <x:c r="D27" s="4"/>
+      <x:c r="E27" s="2"/>
+      <x:c r="F27" s="2"/>
+      <x:c r="G27" s="2"/>
+      <x:c r="H27" s="2"/>
+      <x:c r="I27" s="2"/>
+      <x:c r="J27" s="2"/>
+      <x:c r="K27" s="2"/>
+      <x:c r="L27" s="2"/>
+      <x:c r="M27" s="2"/>
+      <x:c r="N27" s="2"/>
+      <x:c r="O27" s="2"/>
+    </x:row>
+    <x:row r="28" ht="35" customHeight="1">
+      <x:c r="A28" s="4"/>
+      <x:c r="B28" s="4"/>
+      <x:c r="C28" s="4"/>
+      <x:c r="D28" s="4"/>
+      <x:c r="E28" s="2"/>
+      <x:c r="F28" s="2"/>
+      <x:c r="G28" s="2"/>
+      <x:c r="H28" s="2"/>
+      <x:c r="I28" s="2"/>
+      <x:c r="J28" s="2"/>
+      <x:c r="K28" s="2"/>
+      <x:c r="L28" s="2"/>
+      <x:c r="M28" s="2"/>
+      <x:c r="N28" s="2"/>
+      <x:c r="O28" s="2"/>
+    </x:row>
+    <x:row r="29" ht="95" customHeight="1">
+      <x:c r="A29" s="4" t="str">
+        <x:v>Scope / missing history</x:v>
+      </x:c>
+      <x:c r="B29" s="4"/>
+      <x:c r="C29" s="4"/>
+      <x:c r="D29" s="4" t="str">
+        <x:v>Baseline borrowing excludes leases; cash excludes restricted cash and investments. These balances do not establish repayment coverage.</x:v>
+      </x:c>
+      <x:c r="E29" s="2"/>
+      <x:c r="F29" s="2"/>
+      <x:c r="G29" s="2"/>
+      <x:c r="H29" s="2"/>
+      <x:c r="I29" s="2"/>
+      <x:c r="J29" s="2"/>
+      <x:c r="K29" s="2"/>
+      <x:c r="L29" s="2"/>
+      <x:c r="M29" s="2"/>
+      <x:c r="N29" s="2"/>
+      <x:c r="O29" s="2"/>
+    </x:row>
+    <x:row r="30" ht="35" customHeight="1">
+      <x:c r="A30" s="4"/>
+      <x:c r="B30" s="4"/>
+      <x:c r="C30" s="4"/>
+      <x:c r="D30" s="4"/>
+      <x:c r="E30" s="2"/>
+      <x:c r="F30" s="2"/>
+      <x:c r="G30" s="2"/>
+      <x:c r="H30" s="2"/>
+      <x:c r="I30" s="2"/>
+      <x:c r="J30" s="2"/>
+      <x:c r="K30" s="2"/>
+      <x:c r="L30" s="2"/>
+      <x:c r="M30" s="2"/>
+      <x:c r="N30" s="2"/>
+      <x:c r="O30" s="2"/>
+    </x:row>
+    <x:row r="31" ht="35" customHeight="1">
+      <x:c r="A31" s="4"/>
+      <x:c r="B31" s="4"/>
+      <x:c r="C31" s="4"/>
+      <x:c r="D31" s="4"/>
+      <x:c r="E31" s="2"/>
+      <x:c r="F31" s="2"/>
+      <x:c r="G31" s="2"/>
+      <x:c r="H31" s="2"/>
+      <x:c r="I31" s="2"/>
+      <x:c r="J31" s="2"/>
+      <x:c r="K31" s="2"/>
+      <x:c r="L31" s="2"/>
+      <x:c r="M31" s="2"/>
+      <x:c r="N31" s="2"/>
+      <x:c r="O31" s="2"/>
+    </x:row>
+    <x:row r="32" ht="35" customHeight="1">
+      <x:c r="A32" s="4"/>
+      <x:c r="B32" s="4"/>
+      <x:c r="C32" s="4"/>
+      <x:c r="D32" s="4"/>
+      <x:c r="E32" s="2"/>
+      <x:c r="F32" s="2"/>
+      <x:c r="G32" s="2"/>
+      <x:c r="H32" s="2"/>
+      <x:c r="I32" s="2"/>
+      <x:c r="J32" s="2"/>
+      <x:c r="K32" s="2"/>
+      <x:c r="L32" s="2"/>
+      <x:c r="M32" s="2"/>
+      <x:c r="N32" s="2"/>
+      <x:c r="O32" s="2"/>
+    </x:row>
+    <x:row r="33" ht="35" customHeight="1">
+      <x:c r="A33" s="4"/>
+      <x:c r="B33" s="4"/>
+      <x:c r="C33" s="4"/>
+      <x:c r="D33" s="4"/>
+      <x:c r="E33" s="2"/>
+      <x:c r="F33" s="2"/>
+      <x:c r="G33" s="2"/>
+      <x:c r="H33" s="2"/>
+      <x:c r="I33" s="2"/>
+      <x:c r="J33" s="2"/>
+      <x:c r="K33" s="2"/>
+      <x:c r="L33" s="2"/>
+      <x:c r="M33" s="2"/>
+      <x:c r="N33" s="2"/>
+      <x:c r="O33" s="2"/>
+    </x:row>
+    <x:row r="34" ht="35" customHeight="1">
+      <x:c r="A34" s="4"/>
+      <x:c r="B34" s="4"/>
+      <x:c r="C34" s="4"/>
+      <x:c r="D34" s="4"/>
+      <x:c r="E34" s="2"/>
+      <x:c r="F34" s="2"/>
+      <x:c r="G34" s="2"/>
+      <x:c r="H34" s="2"/>
+      <x:c r="I34" s="2"/>
+      <x:c r="J34" s="2"/>
+      <x:c r="K34" s="2"/>
+      <x:c r="L34" s="2"/>
+      <x:c r="M34" s="2"/>
+      <x:c r="N34" s="2"/>
+      <x:c r="O34" s="2"/>
+    </x:row>
+    <x:row r="35" ht="35" customHeight="1">
+      <x:c r="A35" s="4"/>
+      <x:c r="B35" s="4"/>
+      <x:c r="C35" s="4"/>
+      <x:c r="D35" s="4"/>
+      <x:c r="E35" s="2"/>
+      <x:c r="F35" s="2"/>
+      <x:c r="G35" s="2"/>
+      <x:c r="H35" s="2"/>
+      <x:c r="I35" s="2"/>
+      <x:c r="J35" s="2"/>
+      <x:c r="K35" s="2"/>
+      <x:c r="L35" s="2"/>
+      <x:c r="M35" s="2"/>
+      <x:c r="N35" s="2"/>
+      <x:c r="O35" s="2"/>
+    </x:row>
+    <x:row r="36" ht="35" customHeight="1">
+      <x:c r="A36" s="4"/>
+      <x:c r="B36" s="4"/>
+      <x:c r="C36" s="4"/>
+      <x:c r="D36" s="4"/>
+      <x:c r="E36" s="2"/>
+      <x:c r="F36" s="2"/>
+      <x:c r="G36" s="2"/>
+      <x:c r="H36" s="2"/>
+      <x:c r="I36" s="2"/>
+      <x:c r="J36" s="2"/>
+      <x:c r="K36" s="2"/>
+      <x:c r="L36" s="2"/>
+      <x:c r="M36" s="2"/>
+      <x:c r="N36" s="2"/>
+      <x:c r="O36" s="2"/>
+    </x:row>
+    <x:row r="37" ht="35" customHeight="1">
+      <x:c r="A37" s="4"/>
+      <x:c r="B37" s="4"/>
+      <x:c r="C37" s="4"/>
+      <x:c r="D37" s="4"/>
+      <x:c r="E37" s="2"/>
+      <x:c r="F37" s="2"/>
+      <x:c r="G37" s="2"/>
+      <x:c r="H37" s="2"/>
+      <x:c r="I37" s="2"/>
+      <x:c r="J37" s="2"/>
+      <x:c r="K37" s="2"/>
+      <x:c r="L37" s="2"/>
+      <x:c r="M37" s="2"/>
+      <x:c r="N37" s="2"/>
+      <x:c r="O37" s="2"/>
+    </x:row>
+    <x:row r="38" ht="35" customHeight="1">
+      <x:c r="A38" s="4"/>
+      <x:c r="B38" s="4"/>
+      <x:c r="C38" s="4"/>
+      <x:c r="D38" s="4"/>
+      <x:c r="E38" s="2"/>
+      <x:c r="F38" s="2"/>
+      <x:c r="G38" s="2"/>
+      <x:c r="H38" s="2"/>
+      <x:c r="I38" s="2"/>
+      <x:c r="J38" s="2"/>
+      <x:c r="K38" s="2"/>
+      <x:c r="L38" s="2"/>
+      <x:c r="M38" s="2"/>
+      <x:c r="N38" s="2"/>
+      <x:c r="O38" s="2"/>
+    </x:row>
+    <x:row r="39" ht="35" customHeight="1">
+      <x:c r="A39" s="4"/>
+      <x:c r="B39" s="4"/>
+      <x:c r="C39" s="4"/>
+      <x:c r="D39" s="4"/>
+      <x:c r="E39" s="2"/>
+      <x:c r="F39" s="2"/>
+      <x:c r="G39" s="2"/>
+      <x:c r="H39" s="2"/>
+      <x:c r="I39" s="2"/>
+      <x:c r="J39" s="2"/>
+      <x:c r="K39" s="2"/>
+      <x:c r="L39" s="2"/>
+      <x:c r="M39" s="2"/>
+      <x:c r="N39" s="2"/>
+      <x:c r="O39" s="2"/>
+    </x:row>
+    <x:row r="40" ht="35" customHeight="1">
+      <x:c r="A40" s="4"/>
+      <x:c r="B40" s="4"/>
+      <x:c r="C40" s="4"/>
+      <x:c r="D40" s="4"/>
+      <x:c r="E40" s="2"/>
+      <x:c r="F40" s="2"/>
+      <x:c r="G40" s="2"/>
+      <x:c r="H40" s="2"/>
+      <x:c r="I40" s="2"/>
+      <x:c r="J40" s="2"/>
+      <x:c r="K40" s="2"/>
+      <x:c r="L40" s="2"/>
+      <x:c r="M40" s="2"/>
+      <x:c r="N40" s="2"/>
+      <x:c r="O40" s="2"/>
+    </x:row>
+    <x:row r="41" ht="35" customHeight="1">
+      <x:c r="A41" s="4"/>
+      <x:c r="B41" s="4"/>
+      <x:c r="C41" s="4"/>
+      <x:c r="D41" s="4"/>
+      <x:c r="E41" s="2"/>
+      <x:c r="F41" s="2"/>
+      <x:c r="G41" s="2"/>
+      <x:c r="H41" s="2"/>
+      <x:c r="I41" s="2"/>
+      <x:c r="J41" s="2"/>
+      <x:c r="K41" s="2"/>
+      <x:c r="L41" s="2"/>
+      <x:c r="M41" s="2"/>
+      <x:c r="N41" s="2"/>
+      <x:c r="O41" s="2"/>
+    </x:row>
+    <x:row r="42" ht="35" customHeight="1">
+      <x:c r="A42" s="4"/>
+      <x:c r="B42" s="4"/>
+      <x:c r="C42" s="4"/>
+      <x:c r="D42" s="4"/>
+      <x:c r="E42" s="2"/>
+      <x:c r="F42" s="2"/>
+      <x:c r="G42" s="2"/>
+      <x:c r="H42" s="2"/>
+      <x:c r="I42" s="2"/>
+      <x:c r="J42" s="2"/>
+      <x:c r="K42" s="2"/>
+      <x:c r="L42" s="2"/>
+      <x:c r="M42" s="2"/>
+      <x:c r="N42" s="2"/>
+      <x:c r="O42" s="2"/>
+    </x:row>
+    <x:row r="43" ht="35" customHeight="1">
+      <x:c r="A43" s="4"/>
+      <x:c r="B43" s="4"/>
+      <x:c r="C43" s="4"/>
+      <x:c r="D43" s="4"/>
+      <x:c r="E43" s="2"/>
+      <x:c r="F43" s="2"/>
+      <x:c r="G43" s="2"/>
+      <x:c r="H43" s="2"/>
+      <x:c r="I43" s="2"/>
+      <x:c r="J43" s="2"/>
+      <x:c r="K43" s="2"/>
+      <x:c r="L43" s="2"/>
+      <x:c r="M43" s="2"/>
+      <x:c r="N43" s="2"/>
+      <x:c r="O43" s="2"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89ff47f5e478437c"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="46" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
@@ -4260,11 +5552,11 @@
     <x:mergeCell ref="A96:D96"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1ec28f33921480d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79db98eea22941d4"/>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -10466,7 +11758,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -10638,6 +11930,17 @@
         <x:v>https://github.com/jackconnolly1000-ux/sec-filing-research-terminal/blob/main/docs/company_history.md</x:v>
       </x:c>
     </x:row>
+    <x:row r="16" ht="70" customHeight="1">
+      <x:c r="A16" s="218" t="str">
+        <x:v>Core charts</x:v>
+      </x:c>
+      <x:c r="B16" s="219" t="str">
+        <x:v>Two native charts link to Debt and liquidity and History. Signed capital spending is a use; FCF is the result. Unsupported older Vistra borrowing is omitted, never plotted as zero.</x:v>
+      </x:c>
+      <x:c r="C16" s="220" t="str">
+        <x:v>https://github.com/jackconnolly1000-ux/sec-filing-research-terminal/blob/main/docs/core_charts.md</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Align individual Excel guides and dated interpretation with app reviews
</commit_message>
<xml_diff>
--- a/samples/lly_liquidity.xlsx
+++ b/samples/lly_liquidity.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding conclusion" sheetId="1" r:id="R545cd74760084c87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Borrowing and leases" sheetId="2" r:id="R238cedd23ec247d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt and liquidity" sheetId="3" r:id="Rd81cc1e44b5f4b44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="History" sheetId="4" r:id="R36028c37b97841dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core charts" sheetId="5" r:id="Ra3a09e8001d84070"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repayment review" sheetId="6" r:id="Rf3d8710805a74af5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="7" r:id="R1a331d15f7f4430c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="8" r:id="R32f8516f62b34357"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding conclusion" sheetId="1" r:id="R1c6648e8b7ec4225"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Borrowing and leases" sheetId="2" r:id="Rf45888c3a1df4b17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt and liquidity" sheetId="3" r:id="Rc135515193e649c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="History" sheetId="4" r:id="R6ae98e4280914bd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core charts" sheetId="5" r:id="R23a724ea0449445e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repayment review" sheetId="6" r:id="Ra29616e5a8fc4e5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="7" r:id="R7fe6dbf74c584970"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="8" r:id="Rb006a05c25e84490"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1558,7 +1558,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8ebdb1b61a44431d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9c8bf6543f4249c6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1588,7 +1588,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5d1e072ed27a4814"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd0bd32b698ae448f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1623,7 +1623,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb8fd9f5b2b7b470e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rad4eba411b834422"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1956,6 +1956,110 @@
         <x:v>Narrative reflects the checked source snapshot. Editing workbook inputs updates calculations but requires a new review of the narrative.</x:v>
       </x:c>
     </x:row>
+    <x:row r="20" ht="44" customHeight="1">
+      <x:c r="A20" s="13" t="str">
+        <x:v>Workbook contents — select the named tab</x:v>
+      </x:c>
+      <x:c r="B20" s="14" t="str">
+        <x:v>Question / evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="44" customHeight="1">
+      <x:c r="A21" s="15" t="str">
+        <x:v>Funding conclusion</x:v>
+      </x:c>
+      <x:c r="B21" s="16" t="str">
+        <x:v>Start here: obligations, accessible resources, competing uses and decisive unknowns.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="44" customHeight="1">
+      <x:c r="A22" s="15" t="str">
+        <x:v>Borrowing and leases</x:v>
+      </x:c>
+      <x:c r="B22" s="16" t="str">
+        <x:v>Borrowing components, dated lease liabilities and uncommenced commitments, separately.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="44" customHeight="1">
+      <x:c r="A23" s="15" t="str">
+        <x:v>Debt and liquidity</x:v>
+      </x:c>
+      <x:c r="B23" s="16" t="str">
+        <x:v>Latest checked ratios, formulas, periods and company-specific limits.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="44" customHeight="1">
+      <x:c r="A24" s="15" t="str">
+        <x:v>History</x:v>
+      </x:c>
+      <x:c r="B24" s="16" t="str">
+        <x:v>Annual versus latest dated balances; overlapping FY and TTM flows. Unavailable is not zero.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="44" customHeight="1">
+      <x:c r="A25" s="15" t="str">
+        <x:v>Core charts</x:v>
+      </x:c>
+      <x:c r="B25" s="16" t="str">
+        <x:v>What remained after capital spending, and how checked cash/borrowing balances changed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="44" customHeight="1">
+      <x:c r="A26" s="15" t="str">
+        <x:v>Repayment review</x:v>
+      </x:c>
+      <x:c r="B26" s="16" t="str">
+        <x:v>H1 cash uses, conditional commitments, credit evidence and selected May issuance maturities.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="44" customHeight="1">
+      <x:c r="A27" s="15" t="str">
+        <x:v>Data</x:v>
+      </x:c>
+      <x:c r="B27" s="16" t="str">
+        <x:v>Reported inputs with filing dates, accessions, tags, contexts and source URLs; separate evidence blocks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="44" customHeight="1">
+      <x:c r="A28" s="17" t="str">
+        <x:v>About</x:v>
+      </x:c>
+      <x:c r="B28" s="18" t="str">
+        <x:v>Definitions, source scope, missing values, colors and methodology references.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="55" customHeight="1">
+      <x:c r="A30" s="72" t="str">
+        <x:v>Units and dates</x:v>
+      </x:c>
+      <x:c r="B30" s="74" t="str">
+        <x:v>Amounts are stored as whole USD and displayed in millions unless marked x or %. Balance sheets are instants; FY and later TTM are overlapping twelve-month windows.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="55" customHeight="1">
+      <x:c r="A31" s="25" t="str">
+        <x:v>Colors</x:v>
+      </x:c>
+      <x:c r="B31" s="16" t="str">
+        <x:v>Blue numeric cells are reported inputs; green formulas reference other sheets; black formulas calculate within a sheet. Green does not mean favorable or recurring cash.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="55" customHeight="1">
+      <x:c r="A32" s="25" t="str">
+        <x:v>Evidence and uncertainty</x:v>
+      </x:c>
+      <x:c r="B32" s="16" t="str">
+        <x:v>Data contains source URLs and filing metadata. Copy a full URL into a browser to open the source. Unavailable is never zero; capacity and later events do not update balance-sheet cash or borrowing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="55" customHeight="1">
+      <x:c r="A33" s="26" t="str">
+        <x:v>Reading the charts</x:v>
+      </x:c>
+      <x:c r="B33" s="18" t="str">
+        <x:v>FCF is OCF less capital spending, not another cash flow to add. Vistra has no supported older borrowing series. Other existing company-specific charts retain their own dated scope.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2983,7 +3087,7 @@
         <x:v>54908000000</x:v>
       </x:c>
       <x:c r="D7" s="16" t="str">
-        <x:v>Carrying amount of borrowing. Operating/finance leases and commitments are excluded. In this 10-Q, the Note 8 fair-value table's carrying amounts (commercial paper 5,284M plus long-term debt including current portion 49,624M) present the same 54,908M; they are not added.</x:v>
+        <x:v>Carrying borrowing; leases and commitments excluded. Latest column only: In this 10-Q, the Note 8 fair-value table's carrying amounts (commercial paper 5,284M plus long-term debt including current portion 49,624M) present the same 54,908M; they are not added.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="45" customHeight="1">
@@ -3018,7 +3122,7 @@
         <x:v>Total current assets / total current liabilities from one balance sheet. Liabilities include more than borrowing; assets include more than cash.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="45" customHeight="1">
+    <x:row r="10" ht="49" customHeight="1">
       <x:c r="A10" s="25" t="str">
         <x:v>Operating cash flow</x:v>
       </x:c>
@@ -3031,7 +3135,7 @@
         <x:v>28083000000</x:v>
       </x:c>
       <x:c r="D10" s="16" t="str">
-        <x:v>Reported historical OCF; recurrence is not established. Uses FY + current YTD - prior YTD.</x:v>
+        <x:v>Annual column: reported fiscal-year OCF. Latest column only: Reported historical OCF; recurrence is not established. Uses FY + current YTD - prior YTD.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="45" customHeight="1">
@@ -3079,7 +3183,7 @@
         <x:v>0.511455525606469</x:v>
       </x:c>
       <x:c r="D13" s="16" t="str">
-        <x:v>Twelve-month OCF / borrowing at each period end. Prior column uses the fiscal year; later column uses TTM. Not repayment coverage.</x:v>
+        <x:v>Twelve-month flow / borrowing at each period end. Annual column uses FY; latest column uses TTM. Not repayment coverage.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="45" customHeight="1">
@@ -3095,10 +3199,10 @@
         <x:v>0.33128141618707657</x:v>
       </x:c>
       <x:c r="D14" s="16" t="str">
-        <x:v>Twelve-month FCF / borrowing at each period end. Prior column uses the fiscal year; later column uses TTM. Not repayment coverage.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="88" customHeight="1">
+        <x:v>Twelve-month flow / borrowing at each period end. Annual column uses FY; latest column uses TTM. Not repayment coverage.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="49" customHeight="1">
       <x:c r="A15" s="26" t="str">
         <x:v>Historical interest coverage</x:v>
       </x:c>
@@ -3111,7 +3215,7 @@
         <x:v>31.17052826691381</x:v>
       </x:c>
       <x:c r="D15" s="18" t="str">
-        <x:v>FY2025 Note 11 explicitly reports interest on borrowings net of capitalized interest. The interim segment table labels the line interest expense without explicitly stating its capitalization basis. All three amounts are used as reported, before any interest-income offset. Capitalized interest is not added or subtracted; its amount and total interest incurred are Unavailable.</x:v>
+        <x:v>Annual interest is reported net of capitalized interest; the later TTM includes interim expense whose capitalization basis is unstated. Amounts remain as reported.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -3909,11 +4013,15 @@
       <x:c r="N40" s="2"/>
       <x:c r="O40" s="2"/>
     </x:row>
-    <x:row r="41" ht="35" customHeight="1">
-      <x:c r="A41" s="4"/>
+    <x:row r="41" ht="65" customHeight="1">
+      <x:c r="A41" s="4" t="str">
+        <x:v>Evidence trail</x:v>
+      </x:c>
       <x:c r="B41" s="4"/>
       <x:c r="C41" s="4"/>
-      <x:c r="D41" s="4"/>
+      <x:c r="D41" s="4" t="str">
+        <x:v>Chart values link to Debt and liquidity and History. Data retains the exact input periods, tags, accessions and source URLs.</x:v>
+      </x:c>
       <x:c r="E41" s="2"/>
       <x:c r="F41" s="2"/>
       <x:c r="G41" s="2"/>
@@ -3962,7 +4070,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89ff47f5e478437c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dfab275f4374f09"/>
 </x:worksheet>
 </file>
 
@@ -5552,7 +5660,7 @@
     <x:mergeCell ref="A96:D96"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79db98eea22941d4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re356147f3866488b"/>
 </x:worksheet>
 </file>
 
@@ -11941,6 +12049,17 @@
         <x:v>https://github.com/jackconnolly1000-ux/sec-filing-research-terminal/blob/main/docs/core_charts.md</x:v>
       </x:c>
     </x:row>
+    <x:row r="17" ht="76" customHeight="1">
+      <x:c r="A17" s="218" t="str">
+        <x:v>Workbook guide</x:v>
+      </x:c>
+      <x:c r="B17" s="219" t="str">
+        <x:v>The first sheet lists all workbook tabs and their questions. Core metrics, dated history and common charts agree with the app. URLs remain full, copyable source text. Native hyperlink actions are not authored by this spreadsheet runtime.</x:v>
+      </x:c>
+      <x:c r="C17" s="220" t="str">
+        <x:v>https://github.com/jackconnolly1000-ux/sec-filing-research-terminal/blob/main/docs/excel_parity.md</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Complete Release 1 source and app reconciliation
</commit_message>
<xml_diff>
--- a/samples/lly_liquidity.xlsx
+++ b/samples/lly_liquidity.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding conclusion" sheetId="1" r:id="R1c6648e8b7ec4225"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Borrowing and leases" sheetId="2" r:id="Rf45888c3a1df4b17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt and liquidity" sheetId="3" r:id="Rc135515193e649c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="History" sheetId="4" r:id="R6ae98e4280914bd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core charts" sheetId="5" r:id="R23a724ea0449445e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repayment review" sheetId="6" r:id="Ra29616e5a8fc4e5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="7" r:id="R7fe6dbf74c584970"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="8" r:id="Rb006a05c25e84490"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding conclusion" sheetId="1" r:id="R5d8071a01baa4740"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Borrowing and leases" sheetId="2" r:id="Rdb561f41d7664885"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt and liquidity" sheetId="3" r:id="R678973a6daee4721"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="History" sheetId="4" r:id="R61b303ccd30848b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core charts" sheetId="5" r:id="R147af0f1d96f4e26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repayment review" sheetId="6" r:id="R2d31b716f68d4673"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="7" r:id="Re3efeb6e05ad497b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="8" r:id="Rc20a55f23ee44f8d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1558,7 +1558,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9c8bf6543f4249c6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rccfae7a6dcce464b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1588,7 +1588,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd0bd32b698ae448f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R530913a246744b55"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1623,7 +1623,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rad4eba411b834422"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6b2c78017318491a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -4070,7 +4070,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dfab275f4374f09"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3cb24b69ae24fc0"/>
 </x:worksheet>
 </file>
 
@@ -5660,7 +5660,7 @@
     <x:mergeCell ref="A96:D96"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re356147f3866488b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf804cb9b07954525"/>
 </x:worksheet>
 </file>
 
@@ -11252,7 +11252,7 @@
         <x:v>Filing location</x:v>
       </x:c>
       <x:c r="N119" s="96" t="str">
-        <x:v>Unavailable reason</x:v>
+        <x:v>Selection / Unavailable reason</x:v>
       </x:c>
       <x:c r="O119" s="14" t="str">
         <x:v>Reviewed source SHA256</x:v>
@@ -11290,7 +11290,9 @@
       <x:c r="M120" s="107" t="str">
         <x:v>10-Q balance sheet, p. 7</x:v>
       </x:c>
-      <x:c r="N120" s="107" t="str"/>
+      <x:c r="N120" s="107" t="str">
+        <x:v>USD instant at the balance-sheet date, from the latest original 10-K or 10-Q itself</x:v>
+      </x:c>
       <x:c r="O120" s="16" t="str"/>
     </x:row>
     <x:row r="121" ht="78" customHeight="1">
@@ -11325,7 +11327,9 @@
       <x:c r="M121" s="107" t="str">
         <x:v>10-Q balance sheet, p. 7</x:v>
       </x:c>
-      <x:c r="N121" s="107" t="str"/>
+      <x:c r="N121" s="107" t="str">
+        <x:v>USD instant at the balance-sheet date, from the latest original 10-K or 10-Q itself</x:v>
+      </x:c>
       <x:c r="O121" s="16" t="str"/>
     </x:row>
     <x:row r="122" ht="78" customHeight="1">
@@ -11357,7 +11361,7 @@
         <x:v>10-Q balance sheet, p. 7</x:v>
       </x:c>
       <x:c r="N122" s="107" t="str">
-        <x:v>Latest-date lease liabilities Unavailable; no checked amount in the 10-Q.</x:v>
+        <x:v>USD instant at the balance-sheet date, from the latest original 10-K or 10-Q itself Latest-date lease liabilities Unavailable; no checked amount in the 10-Q.</x:v>
       </x:c>
       <x:c r="O122" s="16" t="str"/>
     </x:row>
@@ -11399,7 +11403,9 @@
       <x:c r="M123" s="107" t="str">
         <x:v>10-K Note 10, p. 76</x:v>
       </x:c>
-      <x:c r="N123" s="107" t="str"/>
+      <x:c r="N123" s="107" t="str">
+        <x:v>Exact prefixed tag; exact stated instant; USD; no dimensions; agreeing duplicates.</x:v>
+      </x:c>
       <x:c r="O123" s="16" t="str">
         <x:v>d45f8d1e0945df0b7b30254e96ff8c5dbd1df7d15b17c8ef7399c8e0206b7d7f</x:v>
       </x:c>
@@ -11442,7 +11448,9 @@
       <x:c r="M124" s="107" t="str">
         <x:v>10-K Note 10, p. 76</x:v>
       </x:c>
-      <x:c r="N124" s="107" t="str"/>
+      <x:c r="N124" s="107" t="str">
+        <x:v>Exact prefixed tag; exact stated instant; USD; no dimensions; agreeing duplicates.</x:v>
+      </x:c>
       <x:c r="O124" s="16" t="str">
         <x:v>d45f8d1e0945df0b7b30254e96ff8c5dbd1df7d15b17c8ef7399c8e0206b7d7f</x:v>
       </x:c>
@@ -11476,7 +11484,7 @@
         <x:v>10-Q review; June amount not established</x:v>
       </x:c>
       <x:c r="N125" s="107" t="str">
-        <x:v>No checked June amount. The 10-K describes operating leases only; finance leases are not reported, which is not zero.</x:v>
+        <x:v> No checked June amount. The 10-K describes operating leases only; finance leases are not reported, which is not zero.</x:v>
       </x:c>
       <x:c r="O125" s="16" t="str"/>
     </x:row>
@@ -11509,7 +11517,7 @@
         <x:v>Saved pilot evidence; 10-Q review</x:v>
       </x:c>
       <x:c r="N126" s="109" t="str">
-        <x:v>No checked amount for leases not yet commenced is established in the saved pilot evidence. Unavailable does not mean zero.</x:v>
+        <x:v> No checked amount for leases not yet commenced is established in the saved pilot evidence. Unavailable does not mean zero.</x:v>
       </x:c>
       <x:c r="O126" s="18" t="str"/>
     </x:row>

</xml_diff>

<commit_message>
Group Oracle's dated obligations; link workbook sources
Oracle's principal calendar now sits directly under its dated lease
and purchase payments (oracle_principal_view.py), so near-term
obligations read in one place. Every source URL in the three company
workbooks is now a native hyperlink, added after the build by
add_workbook_hyperlinks.py; guide text updated. Removes known
problem 9. Both were reader obstacles from the Oracle case study.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/lly_liquidity.xlsx
+++ b/samples/lly_liquidity.xlsx
@@ -2049,7 +2049,7 @@
         <x:v>Evidence and uncertainty</x:v>
       </x:c>
       <x:c r="B32" s="16" t="str">
-        <x:v>Data contains source URLs and filing metadata. Copy a full URL into a browser to open the source. Unavailable is never zero; capacity and later events do not update balance-sheet cash or borrowing.</x:v>
+        <x:v>Data contains source URLs and filing metadata. Select a source URL to open it in a browser. Unavailable is never zero; capacity and later events do not update balance-sheet cash or borrowing.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="55" customHeight="1">
@@ -11870,6 +11870,128 @@
       <x:c r="O136" s="18" t="str"/>
     </x:row>
   </x:sheetData>
+  <x:hyperlinks xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+    <x:hyperlink ref="L2" r:id="rIdSource1"/>
+    <x:hyperlink ref="L3" r:id="rIdSource2"/>
+    <x:hyperlink ref="L4" r:id="rIdSource3"/>
+    <x:hyperlink ref="L5" r:id="rIdSource4"/>
+    <x:hyperlink ref="L6" r:id="rIdSource5"/>
+    <x:hyperlink ref="L7" r:id="rIdSource6"/>
+    <x:hyperlink ref="L8" r:id="rIdSource7"/>
+    <x:hyperlink ref="L9" r:id="rIdSource8"/>
+    <x:hyperlink ref="L10" r:id="rIdSource9"/>
+    <x:hyperlink ref="L11" r:id="rIdSource10"/>
+    <x:hyperlink ref="L12" r:id="rIdSource11"/>
+    <x:hyperlink ref="G16" r:id="rIdSource12"/>
+    <x:hyperlink ref="G17" r:id="rIdSource13"/>
+    <x:hyperlink ref="M21" r:id="rIdSource14"/>
+    <x:hyperlink ref="M22" r:id="rIdSource15"/>
+    <x:hyperlink ref="M23" r:id="rIdSource16"/>
+    <x:hyperlink ref="M24" r:id="rIdSource17"/>
+    <x:hyperlink ref="M25" r:id="rIdSource18"/>
+    <x:hyperlink ref="M26" r:id="rIdSource19"/>
+    <x:hyperlink ref="M27" r:id="rIdSource20"/>
+    <x:hyperlink ref="M28" r:id="rIdSource21"/>
+    <x:hyperlink ref="M29" r:id="rIdSource22"/>
+    <x:hyperlink ref="M30" r:id="rIdSource23"/>
+    <x:hyperlink ref="M31" r:id="rIdSource24"/>
+    <x:hyperlink ref="M32" r:id="rIdSource25"/>
+    <x:hyperlink ref="M33" r:id="rIdSource26"/>
+    <x:hyperlink ref="M34" r:id="rIdSource27"/>
+    <x:hyperlink ref="M35" r:id="rIdSource28"/>
+    <x:hyperlink ref="M36" r:id="rIdSource29"/>
+    <x:hyperlink ref="M37" r:id="rIdSource30"/>
+    <x:hyperlink ref="M38" r:id="rIdSource31"/>
+    <x:hyperlink ref="M39" r:id="rIdSource32"/>
+    <x:hyperlink ref="M40" r:id="rIdSource33"/>
+    <x:hyperlink ref="M41" r:id="rIdSource34"/>
+    <x:hyperlink ref="M42" r:id="rIdSource35"/>
+    <x:hyperlink ref="M43" r:id="rIdSource36"/>
+    <x:hyperlink ref="M44" r:id="rIdSource37"/>
+    <x:hyperlink ref="M45" r:id="rIdSource38"/>
+    <x:hyperlink ref="M46" r:id="rIdSource39"/>
+    <x:hyperlink ref="M47" r:id="rIdSource40"/>
+    <x:hyperlink ref="M48" r:id="rIdSource41"/>
+    <x:hyperlink ref="M49" r:id="rIdSource42"/>
+    <x:hyperlink ref="M50" r:id="rIdSource43"/>
+    <x:hyperlink ref="M51" r:id="rIdSource44"/>
+    <x:hyperlink ref="M52" r:id="rIdSource45"/>
+    <x:hyperlink ref="M53" r:id="rIdSource46"/>
+    <x:hyperlink ref="M54" r:id="rIdSource47"/>
+    <x:hyperlink ref="M55" r:id="rIdSource48"/>
+    <x:hyperlink ref="M56" r:id="rIdSource49"/>
+    <x:hyperlink ref="M57" r:id="rIdSource50"/>
+    <x:hyperlink ref="M58" r:id="rIdSource51"/>
+    <x:hyperlink ref="M59" r:id="rIdSource52"/>
+    <x:hyperlink ref="M60" r:id="rIdSource53"/>
+    <x:hyperlink ref="M61" r:id="rIdSource54"/>
+    <x:hyperlink ref="M62" r:id="rIdSource55"/>
+    <x:hyperlink ref="M63" r:id="rIdSource56"/>
+    <x:hyperlink ref="M64" r:id="rIdSource57"/>
+    <x:hyperlink ref="M65" r:id="rIdSource58"/>
+    <x:hyperlink ref="M66" r:id="rIdSource59"/>
+    <x:hyperlink ref="M67" r:id="rIdSource60"/>
+    <x:hyperlink ref="M68" r:id="rIdSource61"/>
+    <x:hyperlink ref="M69" r:id="rIdSource62"/>
+    <x:hyperlink ref="M70" r:id="rIdSource63"/>
+    <x:hyperlink ref="M71" r:id="rIdSource64"/>
+    <x:hyperlink ref="M72" r:id="rIdSource65"/>
+    <x:hyperlink ref="M73" r:id="rIdSource66"/>
+    <x:hyperlink ref="M74" r:id="rIdSource67"/>
+    <x:hyperlink ref="M75" r:id="rIdSource68"/>
+    <x:hyperlink ref="M76" r:id="rIdSource69"/>
+    <x:hyperlink ref="M77" r:id="rIdSource70"/>
+    <x:hyperlink ref="M78" r:id="rIdSource71"/>
+    <x:hyperlink ref="M79" r:id="rIdSource72"/>
+    <x:hyperlink ref="M80" r:id="rIdSource73"/>
+    <x:hyperlink ref="M81" r:id="rIdSource74"/>
+    <x:hyperlink ref="M82" r:id="rIdSource75"/>
+    <x:hyperlink ref="M83" r:id="rIdSource76"/>
+    <x:hyperlink ref="M84" r:id="rIdSource77"/>
+    <x:hyperlink ref="M85" r:id="rIdSource78"/>
+    <x:hyperlink ref="M86" r:id="rIdSource79"/>
+    <x:hyperlink ref="M87" r:id="rIdSource80"/>
+    <x:hyperlink ref="M88" r:id="rIdSource81"/>
+    <x:hyperlink ref="M89" r:id="rIdSource82"/>
+    <x:hyperlink ref="M90" r:id="rIdSource83"/>
+    <x:hyperlink ref="M91" r:id="rIdSource84"/>
+    <x:hyperlink ref="M92" r:id="rIdSource85"/>
+    <x:hyperlink ref="M93" r:id="rIdSource86"/>
+    <x:hyperlink ref="M94" r:id="rIdSource87"/>
+    <x:hyperlink ref="M95" r:id="rIdSource88"/>
+    <x:hyperlink ref="M96" r:id="rIdSource89"/>
+    <x:hyperlink ref="M97" r:id="rIdSource90"/>
+    <x:hyperlink ref="M98" r:id="rIdSource91"/>
+    <x:hyperlink ref="M99" r:id="rIdSource92"/>
+    <x:hyperlink ref="M100" r:id="rIdSource93"/>
+    <x:hyperlink ref="M101" r:id="rIdSource94"/>
+    <x:hyperlink ref="M102" r:id="rIdSource95"/>
+    <x:hyperlink ref="M103" r:id="rIdSource96"/>
+    <x:hyperlink ref="L107" r:id="rIdSource97"/>
+    <x:hyperlink ref="L108" r:id="rIdSource98"/>
+    <x:hyperlink ref="L109" r:id="rIdSource99"/>
+    <x:hyperlink ref="L110" r:id="rIdSource100"/>
+    <x:hyperlink ref="L111" r:id="rIdSource101"/>
+    <x:hyperlink ref="L112" r:id="rIdSource102"/>
+    <x:hyperlink ref="L113" r:id="rIdSource103"/>
+    <x:hyperlink ref="L114" r:id="rIdSource104"/>
+    <x:hyperlink ref="L115" r:id="rIdSource105"/>
+    <x:hyperlink ref="L116" r:id="rIdSource106"/>
+    <x:hyperlink ref="L120" r:id="rIdSource107"/>
+    <x:hyperlink ref="L121" r:id="rIdSource108"/>
+    <x:hyperlink ref="L122" r:id="rIdSource109"/>
+    <x:hyperlink ref="L123" r:id="rIdSource110"/>
+    <x:hyperlink ref="L124" r:id="rIdSource111"/>
+    <x:hyperlink ref="L125" r:id="rIdSource112"/>
+    <x:hyperlink ref="L126" r:id="rIdSource113"/>
+    <x:hyperlink ref="L130" r:id="rIdSource114"/>
+    <x:hyperlink ref="L131" r:id="rIdSource115"/>
+    <x:hyperlink ref="L132" r:id="rIdSource116"/>
+    <x:hyperlink ref="L133" r:id="rIdSource117"/>
+    <x:hyperlink ref="L134" r:id="rIdSource118"/>
+    <x:hyperlink ref="L135" r:id="rIdSource119"/>
+    <x:hyperlink ref="L136" r:id="rIdSource120"/>
+  </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -12062,13 +12184,29 @@
         <x:v>Workbook guide</x:v>
       </x:c>
       <x:c r="B17" s="219" t="str">
-        <x:v>The first sheet lists all workbook tabs and their questions. Core metrics, dated history and common charts agree with the app. URLs remain full, copyable source text. Native hyperlink actions are not authored by this spreadsheet runtime.</x:v>
+        <x:v>The first sheet lists all workbook tabs and their questions. Core metrics, dated history and common charts agree with the app. Source URLs are full text and open as links when selected.</x:v>
       </x:c>
       <x:c r="C17" s="220" t="str">
         <x:v>https://github.com/jackconnolly1000-ux/sec-filing-research-terminal/blob/main/docs/excel_parity.md</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:hyperlinks xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+    <x:hyperlink ref="C2" r:id="rIdSource1"/>
+    <x:hyperlink ref="C4" r:id="rIdSource2"/>
+    <x:hyperlink ref="C5" r:id="rIdSource3"/>
+    <x:hyperlink ref="C6" r:id="rIdSource4"/>
+    <x:hyperlink ref="C7" r:id="rIdSource5"/>
+    <x:hyperlink ref="C8" r:id="rIdSource6"/>
+    <x:hyperlink ref="C9" r:id="rIdSource7"/>
+    <x:hyperlink ref="C10" r:id="rIdSource8"/>
+    <x:hyperlink ref="C11" r:id="rIdSource9"/>
+    <x:hyperlink ref="C13" r:id="rIdSource10"/>
+    <x:hyperlink ref="C14" r:id="rIdSource11"/>
+    <x:hyperlink ref="C15" r:id="rIdSource12"/>
+    <x:hyperlink ref="C16" r:id="rIdSource13"/>
+    <x:hyperlink ref="C17" r:id="rIdSource14"/>
+  </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
</xml_diff>